<commit_message>
Update July fuel-risk inflation trajectory
</commit_message>
<xml_diff>
--- a/assets/06_2026_02_Прогноз.xlsx
+++ b/assets/06_2026_02_Прогноз.xlsx
@@ -1,53 +1,53 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
-  <workbookPr codeName="ЭтаКнига"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ЦБ_Работа\04_Прогноз\_1_Прогноз\_Актуальный прогноз\2026\062026\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{459D2F2E-404B-4147-BFFF-107BDE84CDD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-104" yWindow="-104" windowWidth="22326" windowHeight="13329" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
-  <sheets>
-    <sheet name="Прогноз" sheetId="7" r:id="rId1"/>
-    <sheet name="Прогноз (2)" sheetId="15" r:id="rId2"/>
-    <sheet name="РасчетSaar" sheetId="12" r:id="rId3"/>
-    <sheet name="Корректировки" sheetId="11" r:id="rId4"/>
-    <sheet name="Описания" sheetId="9" state="hidden" r:id="rId5"/>
-    <sheet name="Параметры" sheetId="8" state="hidden" r:id="rId6"/>
-    <sheet name="Лист1" sheetId="13" r:id="rId7"/>
-    <sheet name="for_sa" sheetId="14" r:id="rId8"/>
-  </sheets>
-  <externalReferences>
-    <externalReference r:id="rId9"/>
-  </externalReferences>
-  <definedNames>
-    <definedName name="ExternalData_1" localSheetId="6" hidden="1">Лист1!$A$1:$C$16</definedName>
-    <definedName name="ExternalData_2" localSheetId="6" hidden="1">Лист1!$I$1:$K$185</definedName>
-    <definedName name="рассчитываемБИПЦ">[1]БИПЦ!$D$1</definedName>
-  </definedNames>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
-</workbook>
+<ns0:workbook xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:ns5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:ns6="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:ns7="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ns8="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:ns9="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" ns1:Ignorable="x15 xr xr6 xr10 xr2">
+  <ns0:fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <ns0:workbookPr codeName="ЭтаКнига"/>
+  <ns1:AlternateContent>
+    <ns1:Choice Requires="x15">
+      <ns2:absPath url="C:\ЦБ_Работа\04_Прогноз\_1_Прогноз\_Актуальный прогноз\2026\062026\"/>
+    </ns1:Choice>
+  </ns1:AlternateContent>
+  <ns3:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{459D2F2E-404B-4147-BFFF-107BDE84CDD1}" ns4:coauthVersionLast="47" ns4:coauthVersionMax="47" ns5:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <ns0:bookViews>
+    <ns0:workbookView xWindow="-104" yWindow="-104" windowWidth="22326" windowHeight="13329" ns6:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </ns0:bookViews>
+  <ns0:sheets>
+    <ns0:sheet name="Прогноз" sheetId="7" ns7:id="rId1"/>
+    <ns0:sheet name="Прогноз (2)" sheetId="15" ns7:id="rId2"/>
+    <ns0:sheet name="РасчетSaar" sheetId="12" ns7:id="rId3"/>
+    <ns0:sheet name="Корректировки" sheetId="11" ns7:id="rId4"/>
+    <ns0:sheet name="Описания" sheetId="9" state="hidden" ns7:id="rId5"/>
+    <ns0:sheet name="Параметры" sheetId="8" state="hidden" ns7:id="rId6"/>
+    <ns0:sheet name="Лист1" sheetId="13" ns7:id="rId7"/>
+    <ns0:sheet name="for_sa" sheetId="14" ns7:id="rId8"/>
+  </ns0:sheets>
+  <ns0:externalReferences>
+    <ns0:externalReference ns7:id="rId9"/>
+  </ns0:externalReferences>
+  <ns0:definedNames>
+    <ns0:definedName name="ExternalData_1" localSheetId="6" hidden="1">Лист1!$A$1:$C$16</ns0:definedName>
+    <ns0:definedName name="ExternalData_2" localSheetId="6" hidden="1">Лист1!$I$1:$K$185</ns0:definedName>
+    <ns0:definedName name="рассчитываемБИПЦ">[1]БИПЦ!$D$1</ns0:definedName>
+  </ns0:definedNames>
+  <ns0:calcPr calcId="191029" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
+  <ns0:extLst>
+    <ns0:ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <ns8:workbookPr chartTrackingRefBase="1"/>
+    </ns0:ext>
+    <ns0:ext uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <ns9:calcFeatures>
+        <ns9:feature name="microsoft.com:RD"/>
+        <ns9:feature name="microsoft.com:Single"/>
+        <ns9:feature name="microsoft.com:FV"/>
+        <ns9:feature name="microsoft.com:CNMTM"/>
+        <ns9:feature name="microsoft.com:LET_WF"/>
+        <ns9:feature name="microsoft.com:LAMBDA_WF"/>
+        <ns9:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </ns9:calcFeatures>
+    </ns0:ext>
+  </ns0:extLst>
+</ns0:workbook>
 </file>
 
 <file path=xl/connections.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5671,2025 +5671,2025 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:ns4="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr codeName="Лист1"/>
-  <dimension ref="A1:M93"/>
-  <sheetFormatPr defaultRowHeight="14.4" ns3:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="10.8984375" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.3984375" style="14" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.09765625" style="14" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.296875" style="14" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="11.09765625" style="7" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="9.8984375" style="14" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.69921875" style="14" bestFit="1" customWidth="1"/>
-    <col min="10" max="12" width="8.3984375" style="2" customWidth="1"/>
-    <col min="13" max="13" width="12" style="2" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13" ns3:dyDescent="0.3">
-      <c r="E1" s="38">
-        <v>46181</v>
-      </c>
-      <c r="F1" s="38">
-        <v>46181</v>
-      </c>
-      <c r="G1" s="124">
-        <v>46163</v>
-      </c>
-      <c r="H1" s="124">
-        <v>46163</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" ht="21.9" ns3:dyDescent="0.3">
-      <c r="A2" s="44" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="45">
-        <v>-0.5</v>
-      </c>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="44" t="s">
-        <v>1</v>
-      </c>
-      <c r="F2" s="44" t="s">
-        <v>2</v>
-      </c>
-      <c r="G2" s="45" t="s">
-        <v>1</v>
-      </c>
-      <c r="H2" s="45" t="s">
-        <v>2</v>
-      </c>
-      <c r="I2" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="J2" s="6"/>
-      <c r="K2" s="6"/>
-      <c r="L2" s="6"/>
-      <c r="M2" s="6"/>
-    </row>
-    <row r="3" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A3" s="46">
-        <v>44562</v>
-      </c>
-      <c r="B3" s="47"/>
-      <c r="C3" s="47"/>
-      <c r="D3" s="47"/>
-      <c r="E3" s="109">
-        <v>101.22</v>
-      </c>
-      <c r="F3" s="109">
-        <v>108.84</v>
-      </c>
-      <c r="G3" s="47"/>
-      <c r="H3" s="47"/>
-      <c r="I3" s="5"/>
-      <c r="J3" s="15"/>
-      <c r="K3" s="15"/>
-      <c r="L3" s="15"/>
-      <c r="M3" s="15"/>
-    </row>
-    <row r="4" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A4" s="49">
-        <v>44593</v>
-      </c>
-      <c r="B4" s="47"/>
-      <c r="C4" s="47"/>
-      <c r="D4" s="47"/>
-      <c r="E4" s="109">
-        <v>100.94</v>
-      </c>
-      <c r="F4" s="109">
-        <v>108.73</v>
-      </c>
-      <c r="G4" s="47"/>
-      <c r="H4" s="47"/>
-      <c r="I4" s="5"/>
-      <c r="J4" s="15"/>
-      <c r="K4" s="15"/>
-      <c r="L4" s="15"/>
-      <c r="M4" s="15"/>
-    </row>
-    <row r="5" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A5" s="46">
-        <v>44621</v>
-      </c>
-      <c r="B5" s="47"/>
-      <c r="C5" s="47"/>
-      <c r="D5" s="47"/>
-      <c r="E5" s="109">
-        <v>105.55</v>
-      </c>
-      <c r="F5" s="109">
-        <v>113.28999999999999</v>
-      </c>
-      <c r="G5" s="47"/>
-      <c r="H5" s="47"/>
-      <c r="I5" s="5">
-        <f t="shared" ref="I5:I11" si="0">AVERAGE($E3:$E5)^12/100^11-100</f>
-        <v>35.595184449015164</v>
-      </c>
-      <c r="J5" s="15"/>
-      <c r="K5" s="15"/>
-      <c r="L5" s="15"/>
-      <c r="M5" s="15"/>
-    </row>
-    <row r="6" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A6" s="49">
-        <v>44652</v>
-      </c>
-      <c r="B6" s="47"/>
-      <c r="C6" s="47"/>
-      <c r="D6" s="47"/>
-      <c r="E6" s="109">
-        <v>103.28</v>
-      </c>
-      <c r="F6" s="109">
-        <v>116</v>
-      </c>
-      <c r="G6" s="47"/>
-      <c r="H6" s="47"/>
-      <c r="I6" s="5">
-        <f t="shared" si="0"/>
-        <v>46.8984496892717</v>
-      </c>
-      <c r="J6" s="15"/>
-      <c r="K6" s="15"/>
-      <c r="L6" s="15"/>
-      <c r="M6" s="15"/>
-    </row>
-    <row r="7" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A7" s="46">
-        <v>44682</v>
-      </c>
-      <c r="B7" s="47"/>
-      <c r="C7" s="47"/>
-      <c r="D7" s="47"/>
-      <c r="E7" s="109">
-        <v>100.68</v>
-      </c>
-      <c r="F7" s="109">
-        <v>116.31</v>
-      </c>
-      <c r="G7" s="47"/>
-      <c r="H7" s="47"/>
-      <c r="I7" s="5">
-        <f t="shared" si="0"/>
-        <v>45.425701194734813</v>
-      </c>
-      <c r="J7" s="7"/>
-      <c r="K7" s="7"/>
-      <c r="L7" s="7"/>
-      <c r="M7" s="7"/>
-    </row>
-    <row r="8" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A8" s="49">
-        <v>44713</v>
-      </c>
-      <c r="B8" s="50"/>
-      <c r="C8" s="50"/>
-      <c r="D8" s="50"/>
-      <c r="E8" s="110">
-        <v>99.32</v>
-      </c>
-      <c r="F8" s="110">
-        <v>114.88</v>
-      </c>
-      <c r="G8" s="50"/>
-      <c r="H8" s="50"/>
-      <c r="I8" s="5">
-        <f t="shared" si="0"/>
-        <v>13.938422005549114</v>
-      </c>
-      <c r="J8" s="7"/>
-      <c r="K8" s="7"/>
-      <c r="L8" s="7"/>
-      <c r="M8" s="7"/>
-    </row>
-    <row r="9" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A9" s="46">
-        <v>44743</v>
-      </c>
-      <c r="B9" s="50"/>
-      <c r="C9" s="50"/>
-      <c r="D9" s="50"/>
-      <c r="E9" s="110">
-        <v>99.23</v>
-      </c>
-      <c r="F9" s="110">
-        <v>113.75</v>
-      </c>
-      <c r="G9" s="50"/>
-      <c r="H9" s="50"/>
-      <c r="I9" s="5">
-        <f t="shared" si="0"/>
-        <v>-3.036890517072834</v>
-      </c>
-      <c r="J9" s="7"/>
-      <c r="K9" s="7"/>
-      <c r="L9" s="7"/>
-      <c r="M9" s="7"/>
-    </row>
-    <row r="10" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A10" s="49">
-        <v>44774</v>
-      </c>
-      <c r="B10" s="50"/>
-      <c r="C10" s="50"/>
-      <c r="D10" s="50"/>
-      <c r="E10" s="110">
-        <v>99.43</v>
-      </c>
-      <c r="F10" s="110">
-        <v>112.92</v>
-      </c>
-      <c r="G10" s="50"/>
-      <c r="H10" s="50"/>
-      <c r="I10" s="5">
-        <f t="shared" si="0"/>
-        <v>-7.7873860424702173</v>
-      </c>
-      <c r="J10" s="7"/>
-      <c r="K10" s="7"/>
-      <c r="L10" s="7"/>
-      <c r="M10" s="7"/>
-    </row>
-    <row r="11" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A11" s="46">
-        <v>44805</v>
-      </c>
-      <c r="B11" s="50"/>
-      <c r="C11" s="50"/>
-      <c r="D11" s="50"/>
-      <c r="E11" s="110">
-        <v>100.33</v>
-      </c>
-      <c r="F11" s="110">
-        <v>112.46000000000001</v>
-      </c>
-      <c r="G11" s="50"/>
-      <c r="H11" s="50"/>
-      <c r="I11" s="5">
-        <f t="shared" si="0"/>
-        <v>-3.9660258460593951</v>
-      </c>
-      <c r="J11" s="7"/>
-      <c r="K11" s="7"/>
-      <c r="L11" s="7"/>
-      <c r="M11" s="7"/>
-    </row>
-    <row r="12" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A12" s="49">
-        <v>44835</v>
-      </c>
-      <c r="B12" s="50"/>
-      <c r="C12" s="50"/>
-      <c r="D12" s="50"/>
-      <c r="E12" s="110">
-        <v>100.66</v>
-      </c>
-      <c r="F12" s="110">
-        <v>112.17</v>
-      </c>
-      <c r="G12" s="50"/>
-      <c r="H12" s="50"/>
-      <c r="I12" s="5">
-        <f t="shared" ref="I12:I33" si="1">AVERAGE($E10:$E12)^12/100^11-100</f>
-        <v>1.6929965585857332</v>
-      </c>
-      <c r="J12" s="7"/>
-      <c r="K12" s="7"/>
-      <c r="L12" s="7"/>
-      <c r="M12" s="7"/>
-    </row>
-    <row r="13" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A13" s="46">
-        <v>44866</v>
-      </c>
-      <c r="B13" s="50"/>
-      <c r="C13" s="50"/>
-      <c r="D13" s="50"/>
-      <c r="E13" s="110">
-        <v>100.26</v>
-      </c>
-      <c r="F13" s="110">
-        <v>111.51</v>
-      </c>
-      <c r="G13" s="50"/>
-      <c r="H13" s="50"/>
-      <c r="I13" s="5">
-        <f t="shared" si="1"/>
-        <v>5.1161897881733722</v>
-      </c>
-      <c r="J13" s="7"/>
-      <c r="K13" s="7"/>
-      <c r="L13" s="7"/>
-      <c r="M13" s="7"/>
-    </row>
-    <row r="14" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A14" s="49">
-        <v>44896</v>
-      </c>
-      <c r="B14" s="50"/>
-      <c r="C14" s="50"/>
-      <c r="D14" s="50"/>
-      <c r="E14" s="110">
-        <v>100.57</v>
-      </c>
-      <c r="F14" s="110">
-        <v>111.9</v>
-      </c>
-      <c r="G14" s="50"/>
-      <c r="H14" s="50"/>
-      <c r="I14" s="5">
-        <f t="shared" si="1"/>
-        <v>6.1255330606507243</v>
-      </c>
-      <c r="J14" s="7"/>
-      <c r="K14" s="7"/>
-      <c r="L14" s="7"/>
-      <c r="M14" s="7"/>
-    </row>
-    <row r="15" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A15" s="46">
-        <v>44927</v>
-      </c>
-      <c r="B15" s="50"/>
-      <c r="C15" s="50"/>
-      <c r="D15" s="50"/>
-      <c r="E15" s="110">
-        <v>101.13</v>
-      </c>
-      <c r="F15" s="110">
-        <v>111.8</v>
-      </c>
-      <c r="G15" s="50"/>
-      <c r="H15" s="50"/>
-      <c r="I15" s="5">
-        <f t="shared" si="1"/>
-        <v>8.1279436479058518</v>
-      </c>
-      <c r="J15" s="7"/>
-      <c r="K15" s="7"/>
-      <c r="L15" s="7"/>
-      <c r="M15" s="7"/>
-    </row>
-    <row r="16" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A16" s="49">
-        <v>44958</v>
-      </c>
-      <c r="B16" s="52"/>
-      <c r="C16" s="52"/>
-      <c r="D16" s="52"/>
-      <c r="E16" s="111">
-        <v>100.75</v>
-      </c>
-      <c r="F16" s="111">
-        <v>111.59</v>
-      </c>
-      <c r="G16" s="52"/>
-      <c r="H16" s="52"/>
-      <c r="I16" s="5">
-        <f t="shared" si="1"/>
-        <v>10.252389189890948</v>
-      </c>
-      <c r="J16" s="7"/>
-      <c r="K16" s="7"/>
-      <c r="L16" s="7"/>
-      <c r="M16" s="7"/>
-    </row>
-    <row r="17" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A17" s="46">
-        <v>44986</v>
-      </c>
-      <c r="B17" s="52"/>
-      <c r="C17" s="52"/>
-      <c r="D17" s="52"/>
-      <c r="E17" s="112">
-        <v>100.39</v>
-      </c>
-      <c r="F17" s="111">
-        <v>106.14</v>
-      </c>
-      <c r="G17" s="52"/>
-      <c r="H17" s="52"/>
-      <c r="I17" s="5">
-        <f t="shared" si="1"/>
-        <v>9.4675745363242214</v>
-      </c>
-      <c r="J17" s="7"/>
-      <c r="K17" s="7"/>
-      <c r="L17" s="7"/>
-      <c r="M17" s="7"/>
-    </row>
-    <row r="18" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A18" s="49">
-        <v>45017</v>
-      </c>
-      <c r="B18" s="52"/>
-      <c r="C18" s="52"/>
-      <c r="D18" s="52"/>
-      <c r="E18" s="113">
-        <v>100.72</v>
-      </c>
-      <c r="F18" s="111">
-        <v>103.51</v>
-      </c>
-      <c r="G18" s="52"/>
-      <c r="H18" s="52"/>
-      <c r="I18" s="5">
-        <f t="shared" si="1"/>
-        <v>7.6990210897167941</v>
-      </c>
-      <c r="J18" s="7"/>
-      <c r="K18" s="7"/>
-      <c r="L18" s="7"/>
-      <c r="M18" s="7"/>
-    </row>
-    <row r="19" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A19" s="46">
-        <v>45047</v>
-      </c>
-      <c r="B19" s="52"/>
-      <c r="C19" s="52"/>
-      <c r="D19" s="52"/>
-      <c r="E19" s="113">
-        <v>99.75</v>
-      </c>
-      <c r="F19" s="111">
-        <v>102.55</v>
-      </c>
-      <c r="G19" s="52"/>
-      <c r="H19" s="52"/>
-      <c r="I19" s="5">
-        <f t="shared" si="1"/>
-        <v>3.4947589593967621</v>
-      </c>
-      <c r="J19" s="4"/>
-      <c r="K19" s="4"/>
-      <c r="L19" s="4"/>
-      <c r="M19" s="4"/>
-    </row>
-    <row r="20" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A20" s="49">
-        <v>45078</v>
-      </c>
-      <c r="B20" s="52"/>
-      <c r="C20" s="52"/>
-      <c r="D20" s="52"/>
-      <c r="E20" s="113">
-        <v>100.43</v>
-      </c>
-      <c r="F20" s="111">
-        <v>103.69</v>
-      </c>
-      <c r="G20" s="52"/>
-      <c r="H20" s="52"/>
-      <c r="I20" s="5">
-        <f t="shared" si="1"/>
-        <v>3.6599980288131349</v>
-      </c>
-      <c r="J20" s="7"/>
-      <c r="K20" s="7"/>
-      <c r="L20" s="7"/>
-      <c r="M20" s="7"/>
-    </row>
-    <row r="21" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A21" s="46">
-        <v>45108</v>
-      </c>
-      <c r="B21" s="52"/>
-      <c r="C21" s="52"/>
-      <c r="D21" s="52"/>
-      <c r="E21" s="113">
-        <v>100.5</v>
-      </c>
-      <c r="F21" s="111">
-        <v>105.03</v>
-      </c>
-      <c r="G21" s="52"/>
-      <c r="H21" s="52"/>
-      <c r="I21" s="5">
-        <f t="shared" si="1"/>
-        <v>2.7541668485761903</v>
-      </c>
-      <c r="J21" s="7"/>
-      <c r="K21" s="7"/>
-      <c r="L21" s="7"/>
-      <c r="M21" s="7"/>
-    </row>
-    <row r="22" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A22" s="49">
-        <v>45139</v>
-      </c>
-      <c r="B22" s="52"/>
-      <c r="C22" s="52"/>
-      <c r="D22" s="52"/>
-      <c r="E22" s="113">
-        <v>99.93</v>
-      </c>
-      <c r="F22" s="111">
-        <v>105.56</v>
-      </c>
-      <c r="G22" s="53"/>
-      <c r="H22" s="53"/>
-      <c r="I22" s="5">
-        <f t="shared" si="1"/>
-        <v>3.4947589593967621</v>
-      </c>
-      <c r="J22" s="8"/>
-      <c r="K22" s="8"/>
-      <c r="L22" s="8"/>
-      <c r="M22" s="8"/>
-    </row>
-    <row r="23" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A23" s="46">
-        <v>45170</v>
-      </c>
-      <c r="B23" s="56"/>
-      <c r="C23" s="56"/>
-      <c r="D23" s="56"/>
-      <c r="E23" s="113">
-        <v>101.75</v>
-      </c>
-      <c r="F23" s="111">
-        <v>107.05</v>
-      </c>
-      <c r="G23" s="53"/>
-      <c r="H23" s="53"/>
-      <c r="I23" s="5">
-        <f t="shared" si="1"/>
-        <v>9.0770906435823377</v>
-      </c>
-      <c r="J23" s="8"/>
-      <c r="K23" s="8"/>
-      <c r="L23" s="8"/>
-      <c r="M23" s="8"/>
-    </row>
-    <row r="24" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A24" s="49">
-        <v>45200</v>
-      </c>
-      <c r="B24" s="53">
-        <f>E24-0.5</f>
-        <v>99.96</v>
-      </c>
-      <c r="C24" s="53"/>
-      <c r="D24" s="53"/>
-      <c r="E24" s="113">
-        <v>100.46</v>
-      </c>
-      <c r="F24" s="111">
-        <v>106.84</v>
-      </c>
-      <c r="G24" s="53"/>
-      <c r="H24" s="53"/>
-      <c r="I24" s="5">
-        <f t="shared" si="1"/>
-        <v>8.9039524405937271</v>
-      </c>
-      <c r="J24" s="8"/>
-      <c r="K24" s="8"/>
-      <c r="L24" s="8"/>
-      <c r="M24" s="8"/>
-    </row>
-    <row r="25" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A25" s="46">
-        <v>45231</v>
-      </c>
-      <c r="B25" s="56"/>
-      <c r="C25" s="56"/>
-      <c r="D25" s="56"/>
-      <c r="E25" s="113">
-        <v>100.74</v>
-      </c>
-      <c r="F25" s="111">
-        <v>107.34</v>
-      </c>
-      <c r="G25" s="53"/>
-      <c r="H25" s="56"/>
-      <c r="I25" s="5">
-        <f t="shared" si="1"/>
-        <v>12.459571746567661</v>
-      </c>
-      <c r="J25" s="8"/>
-      <c r="K25" s="8"/>
-      <c r="L25" s="8"/>
-      <c r="M25" s="8"/>
-    </row>
-    <row r="26" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A26" s="49">
-        <v>45261</v>
-      </c>
-      <c r="B26" s="53"/>
-      <c r="C26" s="53"/>
-      <c r="D26" s="53"/>
-      <c r="E26" s="113">
-        <v>100.29</v>
-      </c>
-      <c r="F26" s="111">
-        <v>107.05</v>
-      </c>
-      <c r="G26" s="53"/>
-      <c r="H26" s="53"/>
-      <c r="I26" s="5">
-        <f t="shared" si="1"/>
-        <v>6.1255330606507243</v>
-      </c>
-      <c r="J26" s="8"/>
-      <c r="K26" s="8"/>
-      <c r="L26" s="8"/>
-      <c r="M26" s="8"/>
-    </row>
-    <row r="27" spans="1:13" ht="15" customHeight="1" ns3:dyDescent="0.3">
-      <c r="A27" s="46">
-        <v>45292</v>
-      </c>
-      <c r="B27" s="53"/>
-      <c r="C27" s="53"/>
-      <c r="D27" s="53"/>
-      <c r="E27" s="113">
-        <v>100.87</v>
-      </c>
-      <c r="F27" s="111">
-        <v>106.77</v>
-      </c>
-      <c r="G27" s="53"/>
-      <c r="H27" s="53"/>
-      <c r="I27" s="5">
-        <f t="shared" si="1"/>
-        <v>7.8704026017795172</v>
-      </c>
-      <c r="J27" s="8"/>
-      <c r="K27" s="8"/>
-      <c r="L27" s="8"/>
-      <c r="M27" s="8"/>
-    </row>
-    <row r="28" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A28" s="49">
-        <v>45323</v>
-      </c>
-      <c r="B28" s="53"/>
-      <c r="C28" s="53"/>
-      <c r="D28" s="53"/>
-      <c r="E28" s="113">
-        <v>100.53</v>
-      </c>
-      <c r="F28" s="111">
-        <v>106.54</v>
-      </c>
-      <c r="G28" s="53"/>
-      <c r="H28" s="53"/>
-      <c r="I28" s="5">
-        <f t="shared" si="1"/>
-        <v>6.9734305913095938</v>
-      </c>
-      <c r="J28" s="8"/>
-      <c r="K28" s="8"/>
-      <c r="L28" s="8"/>
-      <c r="M28" s="8"/>
-    </row>
-    <row r="29" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A29" s="46">
-        <v>45352</v>
-      </c>
-      <c r="B29" s="53"/>
-      <c r="C29" s="53"/>
-      <c r="D29" s="53"/>
-      <c r="E29" s="113">
-        <v>100.53</v>
-      </c>
-      <c r="F29" s="111">
-        <v>106.68</v>
-      </c>
-      <c r="G29" s="53"/>
-      <c r="H29" s="53"/>
-      <c r="I29" s="5">
-        <f t="shared" si="1"/>
-        <v>7.9991027537831201</v>
-      </c>
-      <c r="J29" s="8"/>
-      <c r="K29" s="8"/>
-      <c r="L29" s="8"/>
-      <c r="M29" s="8"/>
-    </row>
-    <row r="30" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A30" s="49">
-        <v>45383</v>
-      </c>
-      <c r="B30" s="53"/>
-      <c r="C30" s="53"/>
-      <c r="D30" s="53"/>
-      <c r="E30" s="112">
-        <v>100.38</v>
-      </c>
-      <c r="F30" s="111">
-        <v>106.32</v>
-      </c>
-      <c r="G30" s="53"/>
-      <c r="H30" s="53"/>
-      <c r="I30" s="5">
-        <f t="shared" si="1"/>
-        <v>5.9145235035987298</v>
-      </c>
-      <c r="J30" s="8"/>
-      <c r="K30" s="8"/>
-      <c r="L30" s="8"/>
-      <c r="M30" s="8"/>
-    </row>
-    <row r="31" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A31" s="46">
-        <v>45413</v>
-      </c>
-      <c r="B31" s="53"/>
-      <c r="C31" s="53"/>
-      <c r="D31" s="53"/>
-      <c r="E31" s="112">
-        <v>100.94</v>
-      </c>
-      <c r="F31" s="111">
-        <v>107.59</v>
-      </c>
-      <c r="G31" s="53"/>
-      <c r="H31" s="53"/>
-      <c r="I31" s="5">
-        <f t="shared" si="1"/>
-        <v>7.6562147291127332</v>
-      </c>
-      <c r="J31" s="8"/>
-      <c r="K31" s="8"/>
-      <c r="L31" s="8"/>
-      <c r="M31" s="8"/>
-    </row>
-    <row r="32" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A32" s="49">
-        <v>45444</v>
-      </c>
-      <c r="B32" s="53"/>
-      <c r="C32" s="53"/>
-      <c r="D32" s="53"/>
-      <c r="E32" s="112">
-        <v>100.18</v>
-      </c>
-      <c r="F32" s="111">
-        <v>107.33</v>
-      </c>
-      <c r="G32" s="53"/>
-      <c r="H32" s="53"/>
-      <c r="I32" s="5">
-        <f t="shared" si="1"/>
-        <v>6.1677811864499574</v>
-      </c>
-      <c r="J32" s="8"/>
-      <c r="K32" s="8"/>
-      <c r="L32" s="8"/>
-      <c r="M32" s="8"/>
-    </row>
-    <row r="33" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A33" s="46">
-        <v>45474</v>
-      </c>
-      <c r="B33" s="53"/>
-      <c r="C33" s="53"/>
-      <c r="D33" s="53"/>
-      <c r="E33" s="112">
-        <v>101.07</v>
-      </c>
-      <c r="F33" s="111">
-        <v>107.94</v>
-      </c>
-      <c r="G33" s="53"/>
-      <c r="H33" s="53"/>
-      <c r="I33" s="5">
-        <f t="shared" si="1"/>
-        <v>9.1204146012368454</v>
-      </c>
-      <c r="J33" s="8"/>
-      <c r="K33" s="8"/>
-      <c r="L33" s="8"/>
-      <c r="M33" s="8"/>
-    </row>
-    <row r="34" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A34" s="49">
-        <v>45505</v>
-      </c>
-      <c r="B34" s="53"/>
-      <c r="C34" s="53"/>
-      <c r="D34" s="53"/>
-      <c r="E34" s="113">
-        <v>100.09</v>
-      </c>
-      <c r="F34" s="111">
-        <v>108.1</v>
-      </c>
-      <c r="G34" s="53"/>
-      <c r="H34" s="53"/>
-      <c r="I34" s="5">
-        <f t="shared" ref="I34:I62" si="2">AVERAGE($E32:$E34)^12/100^11-100</f>
-        <v>5.4936577073865607</v>
-      </c>
-      <c r="J34" s="8"/>
-      <c r="K34" s="8"/>
-      <c r="L34" s="8"/>
-      <c r="M34" s="8"/>
-    </row>
-    <row r="35" spans="1:13" ht="14.25" customHeight="1" ns3:dyDescent="0.3">
-      <c r="A35" s="46">
-        <v>45536</v>
-      </c>
-      <c r="B35" s="53"/>
-      <c r="C35" s="53"/>
-      <c r="D35" s="53"/>
-      <c r="E35" s="112">
-        <v>100.62</v>
-      </c>
-      <c r="F35" s="111">
-        <v>106.91</v>
-      </c>
-      <c r="G35" s="53"/>
-      <c r="H35" s="53"/>
-      <c r="I35" s="5">
-        <f t="shared" si="2"/>
-        <v>7.3570066212323866</v>
-      </c>
-      <c r="J35" s="8"/>
-      <c r="K35" s="8"/>
-      <c r="L35" s="8"/>
-      <c r="M35" s="8"/>
-    </row>
-    <row r="36" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A36" s="49">
-        <v>45566</v>
-      </c>
-      <c r="B36" s="53"/>
-      <c r="C36" s="53"/>
-      <c r="D36" s="53"/>
-      <c r="E36" s="113">
-        <v>101.02</v>
-      </c>
-      <c r="F36" s="111">
-        <v>107.49</v>
-      </c>
-      <c r="G36" s="53"/>
-      <c r="H36" s="53"/>
-      <c r="I36" s="5">
-        <f t="shared" si="2"/>
-        <v>7.1437534623089078</v>
-      </c>
-      <c r="J36" s="8"/>
-      <c r="K36" s="8"/>
-      <c r="L36" s="8"/>
-      <c r="M36" s="8"/>
-    </row>
-    <row r="37" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A37" s="64">
-        <v>45597</v>
-      </c>
-      <c r="B37" s="65"/>
-      <c r="C37" s="65"/>
-      <c r="D37" s="65"/>
-      <c r="E37" s="114">
-        <v>101.5</v>
-      </c>
-      <c r="F37" s="115">
-        <v>108.31</v>
-      </c>
-      <c r="G37" s="65"/>
-      <c r="H37" s="65"/>
-      <c r="I37" s="5">
-        <f t="shared" si="2"/>
-        <v>13.308867445393446</v>
-      </c>
-      <c r="J37" s="8"/>
-      <c r="K37" s="8"/>
-      <c r="L37" s="8"/>
-      <c r="M37" s="8"/>
-    </row>
-    <row r="38" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A38" s="49">
-        <v>45627</v>
-      </c>
-      <c r="B38" s="57"/>
-      <c r="C38" s="57"/>
-      <c r="D38" s="57"/>
-      <c r="E38" s="113">
-        <v>100.91</v>
-      </c>
-      <c r="F38" s="111">
-        <v>108.98</v>
-      </c>
-      <c r="G38" s="62"/>
-      <c r="H38" s="57"/>
-      <c r="I38" s="53">
-        <f t="shared" si="2"/>
-        <v>14.616501588558791</v>
-      </c>
-      <c r="J38" s="8"/>
-      <c r="K38" s="8"/>
-      <c r="L38" s="8"/>
-      <c r="M38" s="8"/>
-    </row>
-    <row r="39" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A39" s="59">
-        <v>45658</v>
-      </c>
-      <c r="B39" s="55"/>
-      <c r="C39" s="55"/>
-      <c r="D39" s="55"/>
-      <c r="E39" s="113">
-        <v>100.84</v>
-      </c>
-      <c r="F39" s="113">
-        <v>108.95</v>
-      </c>
-      <c r="G39" s="62"/>
-      <c r="H39" s="62"/>
-      <c r="I39" s="55">
-        <f t="shared" si="2"/>
-        <v>13.803248161387785</v>
-      </c>
-      <c r="J39" s="7"/>
-      <c r="K39" s="7"/>
-      <c r="L39" s="7"/>
-      <c r="M39" s="7"/>
-    </row>
-    <row r="40" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A40" s="60">
-        <v>45689</v>
-      </c>
-      <c r="B40" s="55"/>
-      <c r="C40" s="55"/>
-      <c r="D40" s="55"/>
-      <c r="E40" s="113">
-        <v>101.34</v>
-      </c>
-      <c r="F40" s="113">
-        <v>109.83</v>
-      </c>
-      <c r="G40" s="62"/>
-      <c r="H40" s="62"/>
-      <c r="I40" s="55">
-        <f t="shared" si="2"/>
-        <v>13.084800413622574</v>
-      </c>
-      <c r="J40" s="7"/>
-      <c r="K40" s="7"/>
-      <c r="L40" s="7"/>
-      <c r="M40" s="7"/>
-    </row>
-    <row r="41" spans="1:13" ht="15" thickBot="1" ns3:dyDescent="0.35">
-      <c r="A41" s="71">
-        <v>45717</v>
-      </c>
-      <c r="B41" s="66"/>
-      <c r="C41" s="66"/>
-      <c r="D41" s="66"/>
-      <c r="E41" s="114">
-        <v>100.81</v>
-      </c>
-      <c r="F41" s="114">
-        <v>110.13</v>
-      </c>
-      <c r="G41" s="72"/>
-      <c r="H41" s="72"/>
-      <c r="I41" s="66">
-        <f t="shared" si="2"/>
-        <v>12.637884379001619</v>
-      </c>
-      <c r="J41" s="7"/>
-      <c r="K41" s="7"/>
-      <c r="L41" s="7"/>
-      <c r="M41" s="7"/>
-    </row>
-    <row r="42" spans="1:13" ht="15" thickBot="1" ns3:dyDescent="0.35">
-      <c r="A42" s="78">
-        <v>45748</v>
-      </c>
-      <c r="B42" s="79"/>
-      <c r="C42" s="79"/>
-      <c r="D42" s="79"/>
-      <c r="E42" s="116">
-        <v>100.53</v>
-      </c>
-      <c r="F42" s="116">
-        <v>110.3</v>
-      </c>
-      <c r="G42" s="80"/>
-      <c r="H42" s="80"/>
-      <c r="I42" s="79">
-        <f t="shared" si="2"/>
-        <v>11.262713373249582</v>
-      </c>
-      <c r="J42" s="7"/>
-      <c r="K42" s="7"/>
-      <c r="L42" s="7"/>
-      <c r="M42" s="7"/>
-    </row>
-    <row r="43" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A43" s="74">
-        <v>45778</v>
-      </c>
-      <c r="B43" s="75"/>
-      <c r="C43" s="75"/>
-      <c r="D43" s="75"/>
-      <c r="E43" s="117">
-        <v>99.93</v>
-      </c>
-      <c r="F43" s="117">
-        <v>109.2</v>
-      </c>
-      <c r="G43" s="76"/>
-      <c r="H43" s="76"/>
-      <c r="I43" s="75">
-        <f t="shared" si="2"/>
-        <v>5.1999643920905925</v>
-      </c>
-      <c r="J43" s="7"/>
-      <c r="K43" s="7"/>
-      <c r="L43" s="7"/>
-      <c r="M43" s="7"/>
-    </row>
-    <row r="44" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A44" s="60">
-        <v>45809</v>
-      </c>
-      <c r="B44" s="55"/>
-      <c r="C44" s="55"/>
-      <c r="D44" s="55"/>
-      <c r="E44" s="113">
-        <v>99.96</v>
-      </c>
-      <c r="F44" s="113">
-        <v>108.96</v>
-      </c>
-      <c r="G44" s="62"/>
-      <c r="H44" s="62"/>
-      <c r="I44" s="55">
-        <f t="shared" si="2"/>
-        <v>1.6929965585858326</v>
-      </c>
-      <c r="J44" s="7"/>
-      <c r="K44" s="7"/>
-      <c r="L44" s="7"/>
-      <c r="M44" s="7"/>
-    </row>
-    <row r="45" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A45" s="59">
-        <v>45839</v>
-      </c>
-      <c r="B45" s="55"/>
-      <c r="C45" s="55"/>
-      <c r="D45" s="55"/>
-      <c r="E45" s="113">
-        <v>100.36</v>
-      </c>
-      <c r="F45" s="113">
-        <v>108.19</v>
-      </c>
-      <c r="G45" s="62"/>
-      <c r="H45" s="62"/>
-      <c r="I45" s="55">
-        <f t="shared" si="2"/>
-        <v>1.0045960887180883</v>
-      </c>
-      <c r="J45" s="5"/>
-      <c r="K45" s="5"/>
-      <c r="L45" s="5"/>
-      <c r="M45" s="5"/>
-    </row>
-    <row r="46" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A46" s="60">
-        <v>45870</v>
-      </c>
-      <c r="B46" s="55"/>
-      <c r="C46" s="55"/>
-      <c r="D46" s="55"/>
-      <c r="E46" s="113">
-        <v>99.43</v>
-      </c>
-      <c r="F46" s="113">
-        <v>107.48</v>
-      </c>
-      <c r="G46" s="62"/>
-      <c r="H46" s="62"/>
-      <c r="I46" s="55">
-        <f t="shared" si="2"/>
-        <v>-0.99542937430834399</v>
-      </c>
-      <c r="J46" s="5"/>
-      <c r="K46" s="5"/>
-      <c r="L46" s="5"/>
-      <c r="M46" s="5"/>
-    </row>
-    <row r="47" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A47" s="59">
-        <v>45901</v>
-      </c>
-      <c r="B47" s="55"/>
-      <c r="C47" s="55"/>
-      <c r="D47" s="55"/>
-      <c r="E47" s="113">
-        <v>101</v>
-      </c>
-      <c r="F47" s="113">
-        <v>107.88</v>
-      </c>
-      <c r="G47" s="62"/>
-      <c r="H47" s="62"/>
-      <c r="I47" s="55">
-        <f t="shared" si="2"/>
-        <v>3.2061714591574031</v>
-      </c>
-      <c r="J47" s="5"/>
-      <c r="K47" s="5"/>
-      <c r="L47" s="5"/>
-      <c r="M47" s="5"/>
-    </row>
-    <row r="48" spans="1:13" ht="18.45" customHeight="1" ns3:dyDescent="0.3">
-      <c r="A48" s="60">
-        <v>45931</v>
-      </c>
-      <c r="B48" s="55"/>
-      <c r="C48" s="55"/>
-      <c r="D48" s="55"/>
-      <c r="E48" s="113">
-        <v>100.53</v>
-      </c>
-      <c r="F48" s="113">
-        <v>107.36</v>
-      </c>
-      <c r="G48" s="62"/>
-      <c r="H48" s="62"/>
-      <c r="I48" s="55">
-        <f t="shared" si="2"/>
-        <v>3.9083101131258928</v>
-      </c>
-      <c r="J48" s="5"/>
-      <c r="K48" s="5"/>
-      <c r="L48" s="5"/>
-      <c r="M48" s="5"/>
-    </row>
-    <row r="49" spans="1:13" ht="15" thickBot="1" ns3:dyDescent="0.35">
-      <c r="A49" s="71">
-        <v>45962</v>
-      </c>
-      <c r="B49" s="66"/>
-      <c r="C49" s="55"/>
-      <c r="D49" s="55"/>
-      <c r="E49" s="114">
-        <v>100.15</v>
-      </c>
-      <c r="F49" s="114">
-        <v>105.93</v>
-      </c>
-      <c r="G49" s="72"/>
-      <c r="H49" s="72"/>
-      <c r="I49" s="66">
-        <f t="shared" si="2"/>
-        <v>6.9308886717982716</v>
-      </c>
-      <c r="J49" s="5"/>
-      <c r="K49" s="5"/>
-      <c r="L49" s="5"/>
-      <c r="M49" s="5"/>
-    </row>
-    <row r="50" spans="1:13" ht="15" customHeight="1" thickBot="1" ns3:dyDescent="0.35">
-      <c r="A50" s="78">
-        <v>45992</v>
-      </c>
-      <c r="B50" s="79"/>
-      <c r="C50" s="55"/>
-      <c r="D50" s="55"/>
-      <c r="E50" s="116">
-        <v>100.29</v>
-      </c>
-      <c r="F50" s="116">
-        <v>105.28</v>
-      </c>
-      <c r="G50" s="80"/>
-      <c r="H50" s="80"/>
-      <c r="I50" s="79">
-        <f t="shared" si="2"/>
-        <v>3.949748431031864</v>
-      </c>
-      <c r="J50" s="5"/>
-      <c r="K50" s="5"/>
-      <c r="L50" s="5"/>
-      <c r="M50" s="5"/>
-    </row>
-    <row r="51" spans="1:13" ht="15" thickBot="1" ns3:dyDescent="0.35">
-      <c r="A51" s="74">
-        <v>46023</v>
-      </c>
-      <c r="B51" s="87"/>
-      <c r="C51" s="55">
-        <f t="shared" ref="C51:D57" si="3">E51-100</f>
-        <v>1.6</v>
-      </c>
-      <c r="D51" s="55">
-        <f t="shared" si="3"/>
-        <v>6.07</v>
-      </c>
-      <c r="E51" s="75">
-        <v>101.6</v>
-      </c>
-      <c r="F51" s="75">
-        <f t="shared" ref="F51:F74" si="4">ROUND(PRODUCT(E40:E51)/100^11,2)</f>
-        <v>106.07</v>
-      </c>
-      <c r="G51" s="118">
-        <v>101.6</v>
-      </c>
-      <c r="H51" s="118">
-        <v>106.07</v>
-      </c>
-      <c r="I51" s="79">
-        <f t="shared" si="2"/>
-        <v>8.4722085025153433</v>
-      </c>
-    </row>
-    <row r="52" spans="1:13" ht="15" thickBot="1" ns3:dyDescent="0.35">
-      <c r="A52" s="60">
-        <v>46054</v>
-      </c>
-      <c r="B52" s="56"/>
-      <c r="C52" s="55">
-        <f t="shared" si="3"/>
-        <v>1.1</v>
-      </c>
-      <c r="D52" s="55">
-        <f t="shared" si="3"/>
-        <v>5.82</v>
-      </c>
-      <c r="E52" s="55">
-        <v>101.1</v>
-      </c>
-      <c r="F52" s="55">
-        <f t="shared" si="4"/>
-        <v>105.82</v>
-      </c>
-      <c r="G52" s="107">
-        <v>101.1</v>
-      </c>
-      <c r="H52" s="107">
-        <v>105.82</v>
-      </c>
-      <c r="I52" s="79">
-        <f t="shared" si="2"/>
-        <v>12.637884379001619</v>
-      </c>
-    </row>
-    <row r="53" spans="1:13" ht="15" thickBot="1" ns3:dyDescent="0.35">
-      <c r="A53" s="59">
-        <v>46082</v>
-      </c>
-      <c r="B53" s="56"/>
-      <c r="C53" s="55">
-        <f t="shared" si="3"/>
-        <v>0.54</v>
-      </c>
-      <c r="D53" s="55">
-        <f t="shared" si="3"/>
-        <v>5.54</v>
-      </c>
-      <c r="E53" s="70">
-        <v>100.54</v>
-      </c>
-      <c r="F53" s="55">
-        <f t="shared" si="4"/>
-        <v>105.54</v>
-      </c>
-      <c r="G53" s="107">
-        <v>100.54</v>
-      </c>
-      <c r="H53" s="107">
-        <v>105.54</v>
-      </c>
-      <c r="I53" s="79">
-        <f t="shared" si="2"/>
-        <v>13.758222891107337</v>
-      </c>
-    </row>
-    <row r="54" spans="1:13" ht="15" thickBot="1" ns3:dyDescent="0.35">
-      <c r="A54" s="60">
-        <v>46113</v>
-      </c>
-      <c r="B54" s="56"/>
-      <c r="C54" s="55">
-        <f t="shared" si="3"/>
-        <v>-0.28</v>
-      </c>
-      <c r="D54" s="55">
-        <f t="shared" si="3"/>
-        <v>4.69</v>
-      </c>
-      <c r="E54" s="55">
-        <v>99.72</v>
-      </c>
-      <c r="F54" s="55">
-        <f t="shared" si="4"/>
-        <v>104.69</v>
-      </c>
-      <c r="G54" s="107">
-        <v>99.72</v>
-      </c>
-      <c r="H54" s="107">
-        <v>104.69</v>
-      </c>
-      <c r="I54" s="79">
-        <f t="shared" si="2"/>
-        <v>5.5777080228274372</v>
-      </c>
-    </row>
-    <row r="55" spans="1:13" ht="15" thickBot="1" ns3:dyDescent="0.35">
-      <c r="A55" s="59">
-        <v>46143</v>
-      </c>
-      <c r="B55" s="68"/>
-      <c r="C55" s="55">
-        <f t="shared" si="3"/>
-        <v>0.1</v>
-      </c>
-      <c r="D55" s="55">
-        <f t="shared" si="3"/>
-        <v>4.86</v>
-      </c>
-      <c r="E55" s="55">
-        <v>100.1</v>
-      </c>
-      <c r="F55" s="55">
-        <f t="shared" si="4"/>
-        <v>104.86</v>
-      </c>
-      <c r="G55" s="107">
-        <v>99.9</v>
-      </c>
-      <c r="H55" s="107">
-        <v>104.66</v>
-      </c>
-      <c r="I55" s="79">
-        <f t="shared" si="2"/>
-        <v>1.44954211884</v>
-      </c>
-      <c r="J55" s="42"/>
-      <c r="K55" s="42"/>
-      <c r="L55" s="42"/>
-      <c r="M55" s="42"/>
-    </row>
-    <row r="56" spans="1:13" ht="15" thickBot="1" ns3:dyDescent="0.35">
-      <c r="A56" s="60">
-        <v>46174</v>
-      </c>
-      <c r="B56" s="56"/>
-      <c r="C56" s="55">
-        <f t="shared" si="3"/>
-        <v>0.3</v>
-      </c>
-      <c r="D56" s="55">
-        <f t="shared" si="3"/>
-        <v>5.22</v>
-      </c>
-      <c r="E56" s="55">
-        <v>100.3</v>
-      </c>
-      <c r="F56" s="55">
-        <f t="shared" si="4"/>
-        <v>105.22</v>
-      </c>
-      <c r="G56" s="107">
-        <v>100</v>
-      </c>
-      <c r="H56" s="107">
-        <v>104.7</v>
-      </c>
-      <c r="I56" s="79">
-        <f t="shared" si="2"/>
-        <v>0.481057409268</v>
-      </c>
-      <c r="J56"/>
-      <c r="K56"/>
-      <c r="L56"/>
-      <c r="M56"/>
-    </row>
-    <row r="57" spans="1:13" ht="15" thickBot="1" ns3:dyDescent="0.35">
-      <c r="A57" s="59">
-        <v>46204</v>
-      </c>
-      <c r="B57" s="69"/>
-      <c r="C57" s="55">
-        <f t="shared" si="3"/>
-        <v>-0.15</v>
-      </c>
-      <c r="D57" s="55">
-        <f t="shared" si="3"/>
-        <v>4.69</v>
-      </c>
-      <c r="E57" s="55">
-        <v>99.85</v>
-      </c>
-      <c r="F57" s="55">
-        <f t="shared" si="4"/>
-        <v>104.69</v>
-      </c>
-      <c r="G57" s="107">
-        <v>99.9</v>
-      </c>
-      <c r="H57" s="107">
-        <v>104.22</v>
-      </c>
-      <c r="I57" s="79">
-        <f t="shared" si="2"/>
-        <v>1.00459608872</v>
-      </c>
-      <c r="J57"/>
-      <c r="K57"/>
-      <c r="L57"/>
-      <c r="M57"/>
-    </row>
-    <row r="58" spans="1:13" ht="15" thickBot="1" ns3:dyDescent="0.35">
-      <c r="A58" s="60">
-        <v>46235</v>
-      </c>
-      <c r="B58" s="69"/>
-      <c r="C58" s="69"/>
-      <c r="D58" s="69"/>
-      <c r="E58" s="70">
-        <v>99.8</v>
-      </c>
-      <c r="F58" s="55">
-        <f t="shared" si="4"/>
-        <v>105.08</v>
-      </c>
-      <c r="G58" s="107">
-        <v>99.85</v>
-      </c>
-      <c r="H58" s="107">
-        <v>104.66</v>
-      </c>
-      <c r="I58" s="79">
-        <f t="shared" si="2"/>
-        <v>-0.19981676848</v>
-      </c>
-      <c r="J58"/>
-      <c r="K58"/>
-      <c r="L58"/>
-      <c r="M58"/>
-    </row>
-    <row r="59" spans="1:13" ht="15" thickBot="1" ns3:dyDescent="0.35">
-      <c r="A59" s="59">
-        <v>46266</v>
-      </c>
-      <c r="B59" s="69"/>
-      <c r="C59" s="69"/>
-      <c r="D59" s="69"/>
-      <c r="E59" s="70">
-        <v>100.35</v>
-      </c>
-      <c r="F59" s="55">
-        <f t="shared" si="4"/>
-        <v>104.4</v>
-      </c>
-      <c r="G59" s="107">
-        <v>100.45</v>
-      </c>
-      <c r="H59" s="107">
-        <v>104.09</v>
-      </c>
-      <c r="I59" s="79">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J59"/>
-      <c r="K59"/>
-      <c r="L59"/>
-      <c r="M59"/>
-    </row>
-    <row r="60" spans="1:13" ht="15" thickBot="1" ns3:dyDescent="0.35">
-      <c r="A60" s="60">
-        <v>46296</v>
-      </c>
-      <c r="B60" s="56"/>
-      <c r="C60" s="56"/>
-      <c r="D60" s="56"/>
-      <c r="E60" s="70">
-        <v>101.3</v>
-      </c>
-      <c r="F60" s="55">
-        <f t="shared" si="4"/>
-        <v>105.2</v>
-      </c>
-      <c r="G60" s="107">
-        <v>101.3</v>
-      </c>
-      <c r="H60" s="107">
-        <v>104.88</v>
-      </c>
-      <c r="I60" s="79">
-        <f t="shared" si="2"/>
-        <v>5.95669462245</v>
-      </c>
-      <c r="J60"/>
-      <c r="K60"/>
-      <c r="L60"/>
-      <c r="M60"/>
-    </row>
-    <row r="61" spans="1:13" ht="15" thickBot="1" ns3:dyDescent="0.35">
-      <c r="A61" s="59">
-        <v>46327</v>
-      </c>
-      <c r="B61" s="56"/>
-      <c r="C61" s="56"/>
-      <c r="D61" s="56"/>
-      <c r="E61" s="70">
-        <v>100.25</v>
-      </c>
-      <c r="F61" s="55">
-        <f t="shared" si="4"/>
-        <v>105.3</v>
-      </c>
-      <c r="G61" s="107">
-        <v>100.3</v>
-      </c>
-      <c r="H61" s="107">
-        <v>105.04</v>
-      </c>
-      <c r="I61" s="79">
-        <f t="shared" si="2"/>
-        <v>7.87040260178</v>
-      </c>
-      <c r="J61"/>
-      <c r="K61"/>
-      <c r="L61"/>
-      <c r="M61"/>
-    </row>
-    <row r="62" spans="1:13" ht="15" thickBot="1" ns3:dyDescent="0.35">
-      <c r="A62" s="60">
-        <v>46357</v>
-      </c>
-      <c r="B62" s="56"/>
-      <c r="C62" s="56"/>
-      <c r="D62" s="56"/>
-      <c r="E62" s="70">
-        <v>100.3</v>
-      </c>
-      <c r="F62" s="55">
-        <f t="shared" si="4"/>
-        <v>105.32</v>
-      </c>
-      <c r="G62" s="107">
-        <v>100.35</v>
-      </c>
-      <c r="H62" s="107">
-        <v>105.1</v>
-      </c>
-      <c r="I62" s="79">
-        <f t="shared" si="2"/>
-        <v>7.65621472911</v>
-      </c>
-      <c r="J62"/>
-      <c r="K62"/>
-      <c r="L62"/>
-      <c r="M62"/>
-    </row>
-    <row r="63" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A63" s="59">
-        <v>46388</v>
-      </c>
-      <c r="E63" s="8">
-        <v>100.95</v>
-      </c>
-      <c r="F63" s="55">
-        <f t="shared" si="4"/>
-        <v>104.64</v>
-      </c>
-      <c r="G63" s="31">
-        <v>100.95</v>
-      </c>
-      <c r="H63" s="31">
-        <v>104.43</v>
-      </c>
-      <c r="I63" s="8"/>
-      <c r="J63"/>
-      <c r="K63"/>
-      <c r="L63"/>
-      <c r="M63"/>
-    </row>
-    <row r="64" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A64" s="60">
-        <v>46419</v>
-      </c>
-      <c r="E64" s="8">
-        <v>100.65</v>
-      </c>
-      <c r="F64" s="55">
-        <f t="shared" si="4"/>
-        <v>104.18</v>
-      </c>
-      <c r="G64" s="31">
-        <v>100.65</v>
-      </c>
-      <c r="H64" s="31">
-        <v>103.97</v>
-      </c>
-      <c r="I64" s="8"/>
-      <c r="J64"/>
-      <c r="K64"/>
-      <c r="L64"/>
-      <c r="M64"/>
-    </row>
-    <row r="65" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A65" s="59">
-        <v>46447</v>
-      </c>
-      <c r="E65" s="8">
-        <v>100.5</v>
-      </c>
-      <c r="F65" s="55">
-        <f t="shared" si="4"/>
-        <v>104.13</v>
-      </c>
-      <c r="G65" s="31">
-        <v>100.5</v>
-      </c>
-      <c r="H65" s="31">
-        <v>103.93</v>
-      </c>
-      <c r="I65" s="8"/>
-      <c r="J65"/>
-      <c r="K65"/>
-      <c r="L65"/>
-      <c r="M65"/>
-    </row>
-    <row r="66" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A66" s="60">
-        <v>46478</v>
-      </c>
-      <c r="E66" s="8">
-        <v>100.45</v>
-      </c>
-      <c r="F66" s="55">
-        <f t="shared" si="4"/>
-        <v>104.9</v>
-      </c>
-      <c r="G66" s="31">
-        <v>100.45</v>
-      </c>
-      <c r="H66" s="31">
-        <v>104.69</v>
-      </c>
-      <c r="I66" s="8"/>
-      <c r="J66"/>
-      <c r="K66"/>
-      <c r="L66"/>
-      <c r="M66"/>
-    </row>
-    <row r="67" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A67" s="59">
-        <v>46508</v>
-      </c>
-      <c r="E67" s="8">
-        <v>100.2</v>
-      </c>
-      <c r="F67" s="55">
-        <f t="shared" si="4"/>
-        <v>105</v>
-      </c>
-      <c r="G67" s="31">
-        <v>100.2</v>
-      </c>
-      <c r="H67" s="31">
-        <v>105</v>
-      </c>
-      <c r="I67" s="8"/>
-      <c r="J67"/>
-      <c r="K67"/>
-      <c r="L67"/>
-      <c r="M67"/>
-    </row>
-    <row r="68" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A68" s="60">
-        <v>46539</v>
-      </c>
-      <c r="E68" s="8">
-        <v>100.1</v>
-      </c>
-      <c r="F68" s="55">
-        <f t="shared" si="4"/>
-        <v>104.79</v>
-      </c>
-      <c r="G68" s="31">
-        <v>100.1</v>
-      </c>
-      <c r="H68" s="31">
-        <v>105.11</v>
-      </c>
-      <c r="I68" s="8"/>
-      <c r="J68"/>
-      <c r="K68"/>
-      <c r="L68"/>
-      <c r="M68"/>
-    </row>
-    <row r="69" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A69" s="59">
-        <v>46569</v>
-      </c>
-      <c r="E69" s="8">
-        <v>100.05</v>
-      </c>
-      <c r="F69" s="55">
-        <f t="shared" si="4"/>
-        <v>105</v>
-      </c>
-      <c r="G69" s="31">
-        <v>100.05</v>
-      </c>
-      <c r="H69" s="31">
-        <v>105.26</v>
-      </c>
-      <c r="I69" s="8"/>
-      <c r="J69"/>
-      <c r="K69"/>
-      <c r="L69"/>
-      <c r="M69"/>
-    </row>
-    <row r="70" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A70" s="60">
-        <v>46600</v>
-      </c>
-      <c r="E70" s="8">
-        <v>99.95</v>
-      </c>
-      <c r="F70" s="55">
-        <f t="shared" si="4"/>
-        <v>105.16</v>
-      </c>
-      <c r="G70" s="31">
-        <v>99.95</v>
-      </c>
-      <c r="H70" s="31">
-        <v>105.37</v>
-      </c>
-      <c r="I70" s="8"/>
-      <c r="J70"/>
-      <c r="K70"/>
-      <c r="L70"/>
-      <c r="M70"/>
-    </row>
-    <row r="71" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A71" s="59">
-        <v>46631</v>
-      </c>
-      <c r="E71" s="8">
-        <v>100.45</v>
-      </c>
-      <c r="F71" s="55">
-        <f t="shared" si="4"/>
-        <v>105.26</v>
-      </c>
-      <c r="G71" s="31">
-        <v>100.45</v>
-      </c>
-      <c r="H71" s="31">
-        <v>105.37</v>
-      </c>
-      <c r="I71" s="8"/>
-      <c r="J71"/>
-      <c r="K71"/>
-      <c r="L71"/>
-      <c r="M71"/>
-    </row>
-    <row r="72" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A72" s="60">
-        <v>46661</v>
-      </c>
-      <c r="E72" s="8">
-        <v>100.45</v>
-      </c>
-      <c r="F72" s="55">
-        <f t="shared" si="4"/>
-        <v>104.38</v>
-      </c>
-      <c r="G72" s="31">
-        <v>100.45</v>
-      </c>
-      <c r="H72" s="31">
-        <v>104.49</v>
-      </c>
-      <c r="I72" s="8"/>
-      <c r="J72"/>
-      <c r="K72"/>
-      <c r="L72"/>
-      <c r="M72"/>
-    </row>
-    <row r="73" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A73" s="59">
-        <v>46692</v>
-      </c>
-      <c r="E73" s="8">
-        <v>100.2</v>
-      </c>
-      <c r="F73" s="55">
-        <f t="shared" si="4"/>
-        <v>104.33</v>
-      </c>
-      <c r="G73" s="31">
-        <v>100.2</v>
-      </c>
-      <c r="H73" s="31">
-        <v>104.38</v>
-      </c>
-      <c r="I73" s="8"/>
-      <c r="J73"/>
-      <c r="K73"/>
-      <c r="L73"/>
-      <c r="M73"/>
-    </row>
-    <row r="74" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A74" s="60">
-        <v>46722</v>
-      </c>
-      <c r="E74" s="8">
-        <v>100</v>
-      </c>
-      <c r="F74" s="55">
-        <f t="shared" si="4"/>
-        <v>104.02</v>
-      </c>
-      <c r="G74" s="31">
-        <v>100</v>
-      </c>
-      <c r="H74" s="31">
-        <v>104.02</v>
-      </c>
-      <c r="I74" s="8"/>
-      <c r="J74"/>
-      <c r="K74"/>
-      <c r="L74"/>
-      <c r="M74"/>
-    </row>
-    <row r="75" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A75" s="40"/>
-      <c r="E75" s="22"/>
-      <c r="F75" s="8"/>
-      <c r="G75" s="31"/>
-      <c r="H75" s="31"/>
-      <c r="I75" s="8"/>
-      <c r="J75"/>
-      <c r="K75"/>
-      <c r="L75"/>
-      <c r="M75"/>
-    </row>
-    <row r="76" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A76" s="40"/>
-      <c r="E76" s="22"/>
-      <c r="F76" s="8"/>
-      <c r="G76" s="31"/>
-      <c r="H76" s="31"/>
-      <c r="I76" s="8"/>
-      <c r="J76"/>
-      <c r="K76"/>
-      <c r="L76"/>
-      <c r="M76"/>
-    </row>
-    <row r="77" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A77" s="40"/>
-      <c r="E77" s="22"/>
-      <c r="F77" s="8"/>
-      <c r="G77" s="31"/>
-      <c r="H77" s="31"/>
-      <c r="I77" s="8"/>
-      <c r="J77"/>
-      <c r="K77"/>
-      <c r="L77"/>
-      <c r="M77"/>
-    </row>
-    <row r="78" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A78" s="40"/>
-      <c r="E78" s="22"/>
-      <c r="F78" s="8"/>
-      <c r="G78" s="31"/>
-      <c r="H78" s="31"/>
-      <c r="I78" s="8"/>
-      <c r="J78"/>
-      <c r="K78"/>
-      <c r="L78"/>
-      <c r="M78"/>
-    </row>
-    <row r="79" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A79" s="40"/>
-      <c r="E79" s="22"/>
-      <c r="F79" s="8"/>
-      <c r="G79" s="31"/>
-      <c r="H79" s="31"/>
-      <c r="I79" s="8"/>
-      <c r="J79"/>
-      <c r="K79"/>
-      <c r="L79"/>
-      <c r="M79"/>
-    </row>
-    <row r="80" spans="1:13" ns3:dyDescent="0.3">
-      <c r="A80"/>
-    </row>
-    <row r="81" spans="7:13" ns3:dyDescent="0.3">
-      <c r="G81" s="5"/>
-      <c r="H81" s="5"/>
-      <c r="J81"/>
-      <c r="K81"/>
-      <c r="L81"/>
-      <c r="M81"/>
-    </row>
-    <row r="82" spans="7:13" ns3:dyDescent="0.3">
-      <c r="G82" s="5"/>
-      <c r="H82" s="5"/>
-      <c r="J82"/>
-      <c r="K82"/>
-      <c r="L82"/>
-      <c r="M82"/>
-    </row>
-    <row r="83" spans="7:13" ns3:dyDescent="0.3">
-      <c r="J83"/>
-      <c r="K83"/>
-      <c r="L83"/>
-      <c r="M83"/>
-    </row>
-    <row r="84" spans="7:13" ns3:dyDescent="0.3">
-      <c r="J84"/>
-      <c r="K84"/>
-      <c r="L84"/>
-      <c r="M84"/>
-    </row>
-    <row r="85" spans="7:13" ns3:dyDescent="0.3">
-      <c r="J85"/>
-      <c r="K85"/>
-      <c r="L85"/>
-      <c r="M85"/>
-    </row>
-    <row r="86" spans="7:13" ns3:dyDescent="0.3">
-      <c r="J86"/>
-      <c r="K86"/>
-      <c r="L86"/>
-      <c r="M86"/>
-    </row>
-    <row r="87" spans="7:13" ns3:dyDescent="0.3">
-      <c r="J87"/>
-      <c r="K87"/>
-      <c r="L87"/>
-      <c r="M87"/>
-    </row>
-    <row r="88" spans="7:13" ns3:dyDescent="0.3">
-      <c r="J88"/>
-      <c r="K88"/>
-      <c r="L88"/>
-      <c r="M88"/>
-    </row>
-    <row r="89" spans="7:13" ns3:dyDescent="0.3">
-      <c r="J89"/>
-      <c r="K89"/>
-      <c r="L89"/>
-      <c r="M89"/>
-    </row>
-    <row r="90" spans="7:13" ns3:dyDescent="0.3">
-      <c r="J90"/>
-      <c r="K90"/>
-      <c r="L90"/>
-      <c r="M90"/>
-    </row>
-    <row r="91" spans="7:13" ns3:dyDescent="0.3">
-      <c r="J91"/>
-      <c r="K91"/>
-      <c r="L91"/>
-      <c r="M91"/>
-    </row>
-    <row r="92" spans="7:13" ns3:dyDescent="0.3">
-      <c r="J92"/>
-      <c r="K92"/>
-      <c r="L92"/>
-      <c r="M92"/>
-    </row>
-    <row r="93" spans="7:13" ns3:dyDescent="0.3">
-      <c r="J93"/>
-      <c r="K93"/>
-      <c r="L93"/>
-      <c r="M93"/>
-    </row>
-  </sheetData>
-  <conditionalFormatting sqref="J23:M24">
-    <cfRule type="colorScale" priority="20">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="landscape" ns4:id="rId1"/>
-</worksheet>
+<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:ns4="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
+  <ns0:sheetPr codeName="Лист1"/>
+  <ns0:dimension ref="A1:M93"/>
+  <ns0:sheetFormatPr defaultRowHeight="14.4" ns3:dyDescent="0.3"/>
+  <ns0:cols>
+    <ns0:col min="1" max="1" width="10.8984375" style="3" bestFit="1" customWidth="1"/>
+    <ns0:col min="2" max="2" width="6.3984375" style="14" bestFit="1" customWidth="1"/>
+    <ns0:col min="3" max="3" width="5.09765625" style="14" bestFit="1" customWidth="1"/>
+    <ns0:col min="4" max="4" width="15.296875" style="14" bestFit="1" customWidth="1"/>
+    <ns0:col min="5" max="6" width="11.09765625" style="7" bestFit="1" customWidth="1"/>
+    <ns0:col min="7" max="8" width="9.8984375" style="14" bestFit="1" customWidth="1"/>
+    <ns0:col min="9" max="9" width="6.69921875" style="14" bestFit="1" customWidth="1"/>
+    <ns0:col min="10" max="12" width="8.3984375" style="2" customWidth="1"/>
+    <ns0:col min="13" max="13" width="12" style="2" bestFit="1" customWidth="1"/>
+  </ns0:cols>
+  <ns0:sheetData>
+    <ns0:row r="1" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="E1" s="38">
+        <ns0:v>46181</ns0:v>
+      </ns0:c>
+      <ns0:c r="F1" s="38">
+        <ns0:v>46181</ns0:v>
+      </ns0:c>
+      <ns0:c r="G1" s="124">
+        <ns0:v>46163</ns0:v>
+      </ns0:c>
+      <ns0:c r="H1" s="124">
+        <ns0:v>46163</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="2" spans="1:13" ht="21.9" ns3:dyDescent="0.3">
+      <ns0:c r="A2" s="44" t="s">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="B2" s="45">
+        <ns0:v>-0.5</ns0:v>
+      </ns0:c>
+      <ns0:c r="C2" s="45"/>
+      <ns0:c r="D2" s="45"/>
+      <ns0:c r="E2" s="44" t="s">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+      <ns0:c r="F2" s="44" t="s">
+        <ns0:v>2</ns0:v>
+      </ns0:c>
+      <ns0:c r="G2" s="45" t="s">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+      <ns0:c r="H2" s="45" t="s">
+        <ns0:v>2</ns0:v>
+      </ns0:c>
+      <ns0:c r="I2" s="10" t="s">
+        <ns0:v>32</ns0:v>
+      </ns0:c>
+      <ns0:c r="J2" s="6"/>
+      <ns0:c r="K2" s="6"/>
+      <ns0:c r="L2" s="6"/>
+      <ns0:c r="M2" s="6"/>
+    </ns0:row>
+    <ns0:row r="3" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A3" s="46">
+        <ns0:v>44562</ns0:v>
+      </ns0:c>
+      <ns0:c r="B3" s="47"/>
+      <ns0:c r="C3" s="47"/>
+      <ns0:c r="D3" s="47"/>
+      <ns0:c r="E3" s="109">
+        <ns0:v>101.22</ns0:v>
+      </ns0:c>
+      <ns0:c r="F3" s="109">
+        <ns0:v>108.84</ns0:v>
+      </ns0:c>
+      <ns0:c r="G3" s="47"/>
+      <ns0:c r="H3" s="47"/>
+      <ns0:c r="I3" s="5"/>
+      <ns0:c r="J3" s="15"/>
+      <ns0:c r="K3" s="15"/>
+      <ns0:c r="L3" s="15"/>
+      <ns0:c r="M3" s="15"/>
+    </ns0:row>
+    <ns0:row r="4" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A4" s="49">
+        <ns0:v>44593</ns0:v>
+      </ns0:c>
+      <ns0:c r="B4" s="47"/>
+      <ns0:c r="C4" s="47"/>
+      <ns0:c r="D4" s="47"/>
+      <ns0:c r="E4" s="109">
+        <ns0:v>100.94</ns0:v>
+      </ns0:c>
+      <ns0:c r="F4" s="109">
+        <ns0:v>108.73</ns0:v>
+      </ns0:c>
+      <ns0:c r="G4" s="47"/>
+      <ns0:c r="H4" s="47"/>
+      <ns0:c r="I4" s="5"/>
+      <ns0:c r="J4" s="15"/>
+      <ns0:c r="K4" s="15"/>
+      <ns0:c r="L4" s="15"/>
+      <ns0:c r="M4" s="15"/>
+    </ns0:row>
+    <ns0:row r="5" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A5" s="46">
+        <ns0:v>44621</ns0:v>
+      </ns0:c>
+      <ns0:c r="B5" s="47"/>
+      <ns0:c r="C5" s="47"/>
+      <ns0:c r="D5" s="47"/>
+      <ns0:c r="E5" s="109">
+        <ns0:v>105.55</ns0:v>
+      </ns0:c>
+      <ns0:c r="F5" s="109">
+        <ns0:v>113.28999999999999</ns0:v>
+      </ns0:c>
+      <ns0:c r="G5" s="47"/>
+      <ns0:c r="H5" s="47"/>
+      <ns0:c r="I5" s="5">
+        <ns0:f t="shared" ref="I5:I11" si="0">AVERAGE($E3:$E5)^12/100^11-100</ns0:f>
+        <ns0:v>35.595184449015164</ns0:v>
+      </ns0:c>
+      <ns0:c r="J5" s="15"/>
+      <ns0:c r="K5" s="15"/>
+      <ns0:c r="L5" s="15"/>
+      <ns0:c r="M5" s="15"/>
+    </ns0:row>
+    <ns0:row r="6" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A6" s="49">
+        <ns0:v>44652</ns0:v>
+      </ns0:c>
+      <ns0:c r="B6" s="47"/>
+      <ns0:c r="C6" s="47"/>
+      <ns0:c r="D6" s="47"/>
+      <ns0:c r="E6" s="109">
+        <ns0:v>103.28</ns0:v>
+      </ns0:c>
+      <ns0:c r="F6" s="109">
+        <ns0:v>116</ns0:v>
+      </ns0:c>
+      <ns0:c r="G6" s="47"/>
+      <ns0:c r="H6" s="47"/>
+      <ns0:c r="I6" s="5">
+        <ns0:f t="shared" si="0"/>
+        <ns0:v>46.8984496892717</ns0:v>
+      </ns0:c>
+      <ns0:c r="J6" s="15"/>
+      <ns0:c r="K6" s="15"/>
+      <ns0:c r="L6" s="15"/>
+      <ns0:c r="M6" s="15"/>
+    </ns0:row>
+    <ns0:row r="7" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A7" s="46">
+        <ns0:v>44682</ns0:v>
+      </ns0:c>
+      <ns0:c r="B7" s="47"/>
+      <ns0:c r="C7" s="47"/>
+      <ns0:c r="D7" s="47"/>
+      <ns0:c r="E7" s="109">
+        <ns0:v>100.68</ns0:v>
+      </ns0:c>
+      <ns0:c r="F7" s="109">
+        <ns0:v>116.31</ns0:v>
+      </ns0:c>
+      <ns0:c r="G7" s="47"/>
+      <ns0:c r="H7" s="47"/>
+      <ns0:c r="I7" s="5">
+        <ns0:f t="shared" si="0"/>
+        <ns0:v>45.425701194734813</ns0:v>
+      </ns0:c>
+      <ns0:c r="J7" s="7"/>
+      <ns0:c r="K7" s="7"/>
+      <ns0:c r="L7" s="7"/>
+      <ns0:c r="M7" s="7"/>
+    </ns0:row>
+    <ns0:row r="8" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A8" s="49">
+        <ns0:v>44713</ns0:v>
+      </ns0:c>
+      <ns0:c r="B8" s="50"/>
+      <ns0:c r="C8" s="50"/>
+      <ns0:c r="D8" s="50"/>
+      <ns0:c r="E8" s="110">
+        <ns0:v>99.32</ns0:v>
+      </ns0:c>
+      <ns0:c r="F8" s="110">
+        <ns0:v>114.88</ns0:v>
+      </ns0:c>
+      <ns0:c r="G8" s="50"/>
+      <ns0:c r="H8" s="50"/>
+      <ns0:c r="I8" s="5">
+        <ns0:f t="shared" si="0"/>
+        <ns0:v>13.938422005549114</ns0:v>
+      </ns0:c>
+      <ns0:c r="J8" s="7"/>
+      <ns0:c r="K8" s="7"/>
+      <ns0:c r="L8" s="7"/>
+      <ns0:c r="M8" s="7"/>
+    </ns0:row>
+    <ns0:row r="9" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A9" s="46">
+        <ns0:v>44743</ns0:v>
+      </ns0:c>
+      <ns0:c r="B9" s="50"/>
+      <ns0:c r="C9" s="50"/>
+      <ns0:c r="D9" s="50"/>
+      <ns0:c r="E9" s="110">
+        <ns0:v>99.23</ns0:v>
+      </ns0:c>
+      <ns0:c r="F9" s="110">
+        <ns0:v>113.75</ns0:v>
+      </ns0:c>
+      <ns0:c r="G9" s="50"/>
+      <ns0:c r="H9" s="50"/>
+      <ns0:c r="I9" s="5">
+        <ns0:f t="shared" si="0"/>
+        <ns0:v>-3.036890517072834</ns0:v>
+      </ns0:c>
+      <ns0:c r="J9" s="7"/>
+      <ns0:c r="K9" s="7"/>
+      <ns0:c r="L9" s="7"/>
+      <ns0:c r="M9" s="7"/>
+    </ns0:row>
+    <ns0:row r="10" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A10" s="49">
+        <ns0:v>44774</ns0:v>
+      </ns0:c>
+      <ns0:c r="B10" s="50"/>
+      <ns0:c r="C10" s="50"/>
+      <ns0:c r="D10" s="50"/>
+      <ns0:c r="E10" s="110">
+        <ns0:v>99.43</ns0:v>
+      </ns0:c>
+      <ns0:c r="F10" s="110">
+        <ns0:v>112.92</ns0:v>
+      </ns0:c>
+      <ns0:c r="G10" s="50"/>
+      <ns0:c r="H10" s="50"/>
+      <ns0:c r="I10" s="5">
+        <ns0:f t="shared" si="0"/>
+        <ns0:v>-7.7873860424702173</ns0:v>
+      </ns0:c>
+      <ns0:c r="J10" s="7"/>
+      <ns0:c r="K10" s="7"/>
+      <ns0:c r="L10" s="7"/>
+      <ns0:c r="M10" s="7"/>
+    </ns0:row>
+    <ns0:row r="11" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A11" s="46">
+        <ns0:v>44805</ns0:v>
+      </ns0:c>
+      <ns0:c r="B11" s="50"/>
+      <ns0:c r="C11" s="50"/>
+      <ns0:c r="D11" s="50"/>
+      <ns0:c r="E11" s="110">
+        <ns0:v>100.33</ns0:v>
+      </ns0:c>
+      <ns0:c r="F11" s="110">
+        <ns0:v>112.46000000000001</ns0:v>
+      </ns0:c>
+      <ns0:c r="G11" s="50"/>
+      <ns0:c r="H11" s="50"/>
+      <ns0:c r="I11" s="5">
+        <ns0:f t="shared" si="0"/>
+        <ns0:v>-3.9660258460593951</ns0:v>
+      </ns0:c>
+      <ns0:c r="J11" s="7"/>
+      <ns0:c r="K11" s="7"/>
+      <ns0:c r="L11" s="7"/>
+      <ns0:c r="M11" s="7"/>
+    </ns0:row>
+    <ns0:row r="12" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A12" s="49">
+        <ns0:v>44835</ns0:v>
+      </ns0:c>
+      <ns0:c r="B12" s="50"/>
+      <ns0:c r="C12" s="50"/>
+      <ns0:c r="D12" s="50"/>
+      <ns0:c r="E12" s="110">
+        <ns0:v>100.66</ns0:v>
+      </ns0:c>
+      <ns0:c r="F12" s="110">
+        <ns0:v>112.17</ns0:v>
+      </ns0:c>
+      <ns0:c r="G12" s="50"/>
+      <ns0:c r="H12" s="50"/>
+      <ns0:c r="I12" s="5">
+        <ns0:f t="shared" ref="I12:I33" si="1">AVERAGE($E10:$E12)^12/100^11-100</ns0:f>
+        <ns0:v>1.6929965585857332</ns0:v>
+      </ns0:c>
+      <ns0:c r="J12" s="7"/>
+      <ns0:c r="K12" s="7"/>
+      <ns0:c r="L12" s="7"/>
+      <ns0:c r="M12" s="7"/>
+    </ns0:row>
+    <ns0:row r="13" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A13" s="46">
+        <ns0:v>44866</ns0:v>
+      </ns0:c>
+      <ns0:c r="B13" s="50"/>
+      <ns0:c r="C13" s="50"/>
+      <ns0:c r="D13" s="50"/>
+      <ns0:c r="E13" s="110">
+        <ns0:v>100.26</ns0:v>
+      </ns0:c>
+      <ns0:c r="F13" s="110">
+        <ns0:v>111.51</ns0:v>
+      </ns0:c>
+      <ns0:c r="G13" s="50"/>
+      <ns0:c r="H13" s="50"/>
+      <ns0:c r="I13" s="5">
+        <ns0:f t="shared" si="1"/>
+        <ns0:v>5.1161897881733722</ns0:v>
+      </ns0:c>
+      <ns0:c r="J13" s="7"/>
+      <ns0:c r="K13" s="7"/>
+      <ns0:c r="L13" s="7"/>
+      <ns0:c r="M13" s="7"/>
+    </ns0:row>
+    <ns0:row r="14" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A14" s="49">
+        <ns0:v>44896</ns0:v>
+      </ns0:c>
+      <ns0:c r="B14" s="50"/>
+      <ns0:c r="C14" s="50"/>
+      <ns0:c r="D14" s="50"/>
+      <ns0:c r="E14" s="110">
+        <ns0:v>100.57</ns0:v>
+      </ns0:c>
+      <ns0:c r="F14" s="110">
+        <ns0:v>111.9</ns0:v>
+      </ns0:c>
+      <ns0:c r="G14" s="50"/>
+      <ns0:c r="H14" s="50"/>
+      <ns0:c r="I14" s="5">
+        <ns0:f t="shared" si="1"/>
+        <ns0:v>6.1255330606507243</ns0:v>
+      </ns0:c>
+      <ns0:c r="J14" s="7"/>
+      <ns0:c r="K14" s="7"/>
+      <ns0:c r="L14" s="7"/>
+      <ns0:c r="M14" s="7"/>
+    </ns0:row>
+    <ns0:row r="15" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A15" s="46">
+        <ns0:v>44927</ns0:v>
+      </ns0:c>
+      <ns0:c r="B15" s="50"/>
+      <ns0:c r="C15" s="50"/>
+      <ns0:c r="D15" s="50"/>
+      <ns0:c r="E15" s="110">
+        <ns0:v>101.13</ns0:v>
+      </ns0:c>
+      <ns0:c r="F15" s="110">
+        <ns0:v>111.8</ns0:v>
+      </ns0:c>
+      <ns0:c r="G15" s="50"/>
+      <ns0:c r="H15" s="50"/>
+      <ns0:c r="I15" s="5">
+        <ns0:f t="shared" si="1"/>
+        <ns0:v>8.1279436479058518</ns0:v>
+      </ns0:c>
+      <ns0:c r="J15" s="7"/>
+      <ns0:c r="K15" s="7"/>
+      <ns0:c r="L15" s="7"/>
+      <ns0:c r="M15" s="7"/>
+    </ns0:row>
+    <ns0:row r="16" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A16" s="49">
+        <ns0:v>44958</ns0:v>
+      </ns0:c>
+      <ns0:c r="B16" s="52"/>
+      <ns0:c r="C16" s="52"/>
+      <ns0:c r="D16" s="52"/>
+      <ns0:c r="E16" s="111">
+        <ns0:v>100.75</ns0:v>
+      </ns0:c>
+      <ns0:c r="F16" s="111">
+        <ns0:v>111.59</ns0:v>
+      </ns0:c>
+      <ns0:c r="G16" s="52"/>
+      <ns0:c r="H16" s="52"/>
+      <ns0:c r="I16" s="5">
+        <ns0:f t="shared" si="1"/>
+        <ns0:v>10.252389189890948</ns0:v>
+      </ns0:c>
+      <ns0:c r="J16" s="7"/>
+      <ns0:c r="K16" s="7"/>
+      <ns0:c r="L16" s="7"/>
+      <ns0:c r="M16" s="7"/>
+    </ns0:row>
+    <ns0:row r="17" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A17" s="46">
+        <ns0:v>44986</ns0:v>
+      </ns0:c>
+      <ns0:c r="B17" s="52"/>
+      <ns0:c r="C17" s="52"/>
+      <ns0:c r="D17" s="52"/>
+      <ns0:c r="E17" s="112">
+        <ns0:v>100.39</ns0:v>
+      </ns0:c>
+      <ns0:c r="F17" s="111">
+        <ns0:v>106.14</ns0:v>
+      </ns0:c>
+      <ns0:c r="G17" s="52"/>
+      <ns0:c r="H17" s="52"/>
+      <ns0:c r="I17" s="5">
+        <ns0:f t="shared" si="1"/>
+        <ns0:v>9.4675745363242214</ns0:v>
+      </ns0:c>
+      <ns0:c r="J17" s="7"/>
+      <ns0:c r="K17" s="7"/>
+      <ns0:c r="L17" s="7"/>
+      <ns0:c r="M17" s="7"/>
+    </ns0:row>
+    <ns0:row r="18" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A18" s="49">
+        <ns0:v>45017</ns0:v>
+      </ns0:c>
+      <ns0:c r="B18" s="52"/>
+      <ns0:c r="C18" s="52"/>
+      <ns0:c r="D18" s="52"/>
+      <ns0:c r="E18" s="113">
+        <ns0:v>100.72</ns0:v>
+      </ns0:c>
+      <ns0:c r="F18" s="111">
+        <ns0:v>103.51</ns0:v>
+      </ns0:c>
+      <ns0:c r="G18" s="52"/>
+      <ns0:c r="H18" s="52"/>
+      <ns0:c r="I18" s="5">
+        <ns0:f t="shared" si="1"/>
+        <ns0:v>7.6990210897167941</ns0:v>
+      </ns0:c>
+      <ns0:c r="J18" s="7"/>
+      <ns0:c r="K18" s="7"/>
+      <ns0:c r="L18" s="7"/>
+      <ns0:c r="M18" s="7"/>
+    </ns0:row>
+    <ns0:row r="19" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A19" s="46">
+        <ns0:v>45047</ns0:v>
+      </ns0:c>
+      <ns0:c r="B19" s="52"/>
+      <ns0:c r="C19" s="52"/>
+      <ns0:c r="D19" s="52"/>
+      <ns0:c r="E19" s="113">
+        <ns0:v>99.75</ns0:v>
+      </ns0:c>
+      <ns0:c r="F19" s="111">
+        <ns0:v>102.55</ns0:v>
+      </ns0:c>
+      <ns0:c r="G19" s="52"/>
+      <ns0:c r="H19" s="52"/>
+      <ns0:c r="I19" s="5">
+        <ns0:f t="shared" si="1"/>
+        <ns0:v>3.4947589593967621</ns0:v>
+      </ns0:c>
+      <ns0:c r="J19" s="4"/>
+      <ns0:c r="K19" s="4"/>
+      <ns0:c r="L19" s="4"/>
+      <ns0:c r="M19" s="4"/>
+    </ns0:row>
+    <ns0:row r="20" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A20" s="49">
+        <ns0:v>45078</ns0:v>
+      </ns0:c>
+      <ns0:c r="B20" s="52"/>
+      <ns0:c r="C20" s="52"/>
+      <ns0:c r="D20" s="52"/>
+      <ns0:c r="E20" s="113">
+        <ns0:v>100.43</ns0:v>
+      </ns0:c>
+      <ns0:c r="F20" s="111">
+        <ns0:v>103.69</ns0:v>
+      </ns0:c>
+      <ns0:c r="G20" s="52"/>
+      <ns0:c r="H20" s="52"/>
+      <ns0:c r="I20" s="5">
+        <ns0:f t="shared" si="1"/>
+        <ns0:v>3.6599980288131349</ns0:v>
+      </ns0:c>
+      <ns0:c r="J20" s="7"/>
+      <ns0:c r="K20" s="7"/>
+      <ns0:c r="L20" s="7"/>
+      <ns0:c r="M20" s="7"/>
+    </ns0:row>
+    <ns0:row r="21" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A21" s="46">
+        <ns0:v>45108</ns0:v>
+      </ns0:c>
+      <ns0:c r="B21" s="52"/>
+      <ns0:c r="C21" s="52"/>
+      <ns0:c r="D21" s="52"/>
+      <ns0:c r="E21" s="113">
+        <ns0:v>100.5</ns0:v>
+      </ns0:c>
+      <ns0:c r="F21" s="111">
+        <ns0:v>105.03</ns0:v>
+      </ns0:c>
+      <ns0:c r="G21" s="52"/>
+      <ns0:c r="H21" s="52"/>
+      <ns0:c r="I21" s="5">
+        <ns0:f t="shared" si="1"/>
+        <ns0:v>2.7541668485761903</ns0:v>
+      </ns0:c>
+      <ns0:c r="J21" s="7"/>
+      <ns0:c r="K21" s="7"/>
+      <ns0:c r="L21" s="7"/>
+      <ns0:c r="M21" s="7"/>
+    </ns0:row>
+    <ns0:row r="22" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A22" s="49">
+        <ns0:v>45139</ns0:v>
+      </ns0:c>
+      <ns0:c r="B22" s="52"/>
+      <ns0:c r="C22" s="52"/>
+      <ns0:c r="D22" s="52"/>
+      <ns0:c r="E22" s="113">
+        <ns0:v>99.93</ns0:v>
+      </ns0:c>
+      <ns0:c r="F22" s="111">
+        <ns0:v>105.56</ns0:v>
+      </ns0:c>
+      <ns0:c r="G22" s="53"/>
+      <ns0:c r="H22" s="53"/>
+      <ns0:c r="I22" s="5">
+        <ns0:f t="shared" si="1"/>
+        <ns0:v>3.4947589593967621</ns0:v>
+      </ns0:c>
+      <ns0:c r="J22" s="8"/>
+      <ns0:c r="K22" s="8"/>
+      <ns0:c r="L22" s="8"/>
+      <ns0:c r="M22" s="8"/>
+    </ns0:row>
+    <ns0:row r="23" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A23" s="46">
+        <ns0:v>45170</ns0:v>
+      </ns0:c>
+      <ns0:c r="B23" s="56"/>
+      <ns0:c r="C23" s="56"/>
+      <ns0:c r="D23" s="56"/>
+      <ns0:c r="E23" s="113">
+        <ns0:v>101.75</ns0:v>
+      </ns0:c>
+      <ns0:c r="F23" s="111">
+        <ns0:v>107.05</ns0:v>
+      </ns0:c>
+      <ns0:c r="G23" s="53"/>
+      <ns0:c r="H23" s="53"/>
+      <ns0:c r="I23" s="5">
+        <ns0:f t="shared" si="1"/>
+        <ns0:v>9.0770906435823377</ns0:v>
+      </ns0:c>
+      <ns0:c r="J23" s="8"/>
+      <ns0:c r="K23" s="8"/>
+      <ns0:c r="L23" s="8"/>
+      <ns0:c r="M23" s="8"/>
+    </ns0:row>
+    <ns0:row r="24" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A24" s="49">
+        <ns0:v>45200</ns0:v>
+      </ns0:c>
+      <ns0:c r="B24" s="53">
+        <ns0:f>E24-0.5</ns0:f>
+        <ns0:v>99.96</ns0:v>
+      </ns0:c>
+      <ns0:c r="C24" s="53"/>
+      <ns0:c r="D24" s="53"/>
+      <ns0:c r="E24" s="113">
+        <ns0:v>100.46</ns0:v>
+      </ns0:c>
+      <ns0:c r="F24" s="111">
+        <ns0:v>106.84</ns0:v>
+      </ns0:c>
+      <ns0:c r="G24" s="53"/>
+      <ns0:c r="H24" s="53"/>
+      <ns0:c r="I24" s="5">
+        <ns0:f t="shared" si="1"/>
+        <ns0:v>8.9039524405937271</ns0:v>
+      </ns0:c>
+      <ns0:c r="J24" s="8"/>
+      <ns0:c r="K24" s="8"/>
+      <ns0:c r="L24" s="8"/>
+      <ns0:c r="M24" s="8"/>
+    </ns0:row>
+    <ns0:row r="25" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A25" s="46">
+        <ns0:v>45231</ns0:v>
+      </ns0:c>
+      <ns0:c r="B25" s="56"/>
+      <ns0:c r="C25" s="56"/>
+      <ns0:c r="D25" s="56"/>
+      <ns0:c r="E25" s="113">
+        <ns0:v>100.74</ns0:v>
+      </ns0:c>
+      <ns0:c r="F25" s="111">
+        <ns0:v>107.34</ns0:v>
+      </ns0:c>
+      <ns0:c r="G25" s="53"/>
+      <ns0:c r="H25" s="56"/>
+      <ns0:c r="I25" s="5">
+        <ns0:f t="shared" si="1"/>
+        <ns0:v>12.459571746567661</ns0:v>
+      </ns0:c>
+      <ns0:c r="J25" s="8"/>
+      <ns0:c r="K25" s="8"/>
+      <ns0:c r="L25" s="8"/>
+      <ns0:c r="M25" s="8"/>
+    </ns0:row>
+    <ns0:row r="26" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A26" s="49">
+        <ns0:v>45261</ns0:v>
+      </ns0:c>
+      <ns0:c r="B26" s="53"/>
+      <ns0:c r="C26" s="53"/>
+      <ns0:c r="D26" s="53"/>
+      <ns0:c r="E26" s="113">
+        <ns0:v>100.29</ns0:v>
+      </ns0:c>
+      <ns0:c r="F26" s="111">
+        <ns0:v>107.05</ns0:v>
+      </ns0:c>
+      <ns0:c r="G26" s="53"/>
+      <ns0:c r="H26" s="53"/>
+      <ns0:c r="I26" s="5">
+        <ns0:f t="shared" si="1"/>
+        <ns0:v>6.1255330606507243</ns0:v>
+      </ns0:c>
+      <ns0:c r="J26" s="8"/>
+      <ns0:c r="K26" s="8"/>
+      <ns0:c r="L26" s="8"/>
+      <ns0:c r="M26" s="8"/>
+    </ns0:row>
+    <ns0:row r="27" spans="1:13" ht="15" customHeight="1" ns3:dyDescent="0.3">
+      <ns0:c r="A27" s="46">
+        <ns0:v>45292</ns0:v>
+      </ns0:c>
+      <ns0:c r="B27" s="53"/>
+      <ns0:c r="C27" s="53"/>
+      <ns0:c r="D27" s="53"/>
+      <ns0:c r="E27" s="113">
+        <ns0:v>100.87</ns0:v>
+      </ns0:c>
+      <ns0:c r="F27" s="111">
+        <ns0:v>106.77</ns0:v>
+      </ns0:c>
+      <ns0:c r="G27" s="53"/>
+      <ns0:c r="H27" s="53"/>
+      <ns0:c r="I27" s="5">
+        <ns0:f t="shared" si="1"/>
+        <ns0:v>7.8704026017795172</ns0:v>
+      </ns0:c>
+      <ns0:c r="J27" s="8"/>
+      <ns0:c r="K27" s="8"/>
+      <ns0:c r="L27" s="8"/>
+      <ns0:c r="M27" s="8"/>
+    </ns0:row>
+    <ns0:row r="28" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A28" s="49">
+        <ns0:v>45323</ns0:v>
+      </ns0:c>
+      <ns0:c r="B28" s="53"/>
+      <ns0:c r="C28" s="53"/>
+      <ns0:c r="D28" s="53"/>
+      <ns0:c r="E28" s="113">
+        <ns0:v>100.53</ns0:v>
+      </ns0:c>
+      <ns0:c r="F28" s="111">
+        <ns0:v>106.54</ns0:v>
+      </ns0:c>
+      <ns0:c r="G28" s="53"/>
+      <ns0:c r="H28" s="53"/>
+      <ns0:c r="I28" s="5">
+        <ns0:f t="shared" si="1"/>
+        <ns0:v>6.9734305913095938</ns0:v>
+      </ns0:c>
+      <ns0:c r="J28" s="8"/>
+      <ns0:c r="K28" s="8"/>
+      <ns0:c r="L28" s="8"/>
+      <ns0:c r="M28" s="8"/>
+    </ns0:row>
+    <ns0:row r="29" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A29" s="46">
+        <ns0:v>45352</ns0:v>
+      </ns0:c>
+      <ns0:c r="B29" s="53"/>
+      <ns0:c r="C29" s="53"/>
+      <ns0:c r="D29" s="53"/>
+      <ns0:c r="E29" s="113">
+        <ns0:v>100.53</ns0:v>
+      </ns0:c>
+      <ns0:c r="F29" s="111">
+        <ns0:v>106.68</ns0:v>
+      </ns0:c>
+      <ns0:c r="G29" s="53"/>
+      <ns0:c r="H29" s="53"/>
+      <ns0:c r="I29" s="5">
+        <ns0:f t="shared" si="1"/>
+        <ns0:v>7.9991027537831201</ns0:v>
+      </ns0:c>
+      <ns0:c r="J29" s="8"/>
+      <ns0:c r="K29" s="8"/>
+      <ns0:c r="L29" s="8"/>
+      <ns0:c r="M29" s="8"/>
+    </ns0:row>
+    <ns0:row r="30" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A30" s="49">
+        <ns0:v>45383</ns0:v>
+      </ns0:c>
+      <ns0:c r="B30" s="53"/>
+      <ns0:c r="C30" s="53"/>
+      <ns0:c r="D30" s="53"/>
+      <ns0:c r="E30" s="112">
+        <ns0:v>100.38</ns0:v>
+      </ns0:c>
+      <ns0:c r="F30" s="111">
+        <ns0:v>106.32</ns0:v>
+      </ns0:c>
+      <ns0:c r="G30" s="53"/>
+      <ns0:c r="H30" s="53"/>
+      <ns0:c r="I30" s="5">
+        <ns0:f t="shared" si="1"/>
+        <ns0:v>5.9145235035987298</ns0:v>
+      </ns0:c>
+      <ns0:c r="J30" s="8"/>
+      <ns0:c r="K30" s="8"/>
+      <ns0:c r="L30" s="8"/>
+      <ns0:c r="M30" s="8"/>
+    </ns0:row>
+    <ns0:row r="31" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A31" s="46">
+        <ns0:v>45413</ns0:v>
+      </ns0:c>
+      <ns0:c r="B31" s="53"/>
+      <ns0:c r="C31" s="53"/>
+      <ns0:c r="D31" s="53"/>
+      <ns0:c r="E31" s="112">
+        <ns0:v>100.94</ns0:v>
+      </ns0:c>
+      <ns0:c r="F31" s="111">
+        <ns0:v>107.59</ns0:v>
+      </ns0:c>
+      <ns0:c r="G31" s="53"/>
+      <ns0:c r="H31" s="53"/>
+      <ns0:c r="I31" s="5">
+        <ns0:f t="shared" si="1"/>
+        <ns0:v>7.6562147291127332</ns0:v>
+      </ns0:c>
+      <ns0:c r="J31" s="8"/>
+      <ns0:c r="K31" s="8"/>
+      <ns0:c r="L31" s="8"/>
+      <ns0:c r="M31" s="8"/>
+    </ns0:row>
+    <ns0:row r="32" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A32" s="49">
+        <ns0:v>45444</ns0:v>
+      </ns0:c>
+      <ns0:c r="B32" s="53"/>
+      <ns0:c r="C32" s="53"/>
+      <ns0:c r="D32" s="53"/>
+      <ns0:c r="E32" s="112">
+        <ns0:v>100.18</ns0:v>
+      </ns0:c>
+      <ns0:c r="F32" s="111">
+        <ns0:v>107.33</ns0:v>
+      </ns0:c>
+      <ns0:c r="G32" s="53"/>
+      <ns0:c r="H32" s="53"/>
+      <ns0:c r="I32" s="5">
+        <ns0:f t="shared" si="1"/>
+        <ns0:v>6.1677811864499574</ns0:v>
+      </ns0:c>
+      <ns0:c r="J32" s="8"/>
+      <ns0:c r="K32" s="8"/>
+      <ns0:c r="L32" s="8"/>
+      <ns0:c r="M32" s="8"/>
+    </ns0:row>
+    <ns0:row r="33" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A33" s="46">
+        <ns0:v>45474</ns0:v>
+      </ns0:c>
+      <ns0:c r="B33" s="53"/>
+      <ns0:c r="C33" s="53"/>
+      <ns0:c r="D33" s="53"/>
+      <ns0:c r="E33" s="112">
+        <ns0:v>101.07</ns0:v>
+      </ns0:c>
+      <ns0:c r="F33" s="111">
+        <ns0:v>107.94</ns0:v>
+      </ns0:c>
+      <ns0:c r="G33" s="53"/>
+      <ns0:c r="H33" s="53"/>
+      <ns0:c r="I33" s="5">
+        <ns0:f t="shared" si="1"/>
+        <ns0:v>9.1204146012368454</ns0:v>
+      </ns0:c>
+      <ns0:c r="J33" s="8"/>
+      <ns0:c r="K33" s="8"/>
+      <ns0:c r="L33" s="8"/>
+      <ns0:c r="M33" s="8"/>
+    </ns0:row>
+    <ns0:row r="34" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A34" s="49">
+        <ns0:v>45505</ns0:v>
+      </ns0:c>
+      <ns0:c r="B34" s="53"/>
+      <ns0:c r="C34" s="53"/>
+      <ns0:c r="D34" s="53"/>
+      <ns0:c r="E34" s="113">
+        <ns0:v>100.09</ns0:v>
+      </ns0:c>
+      <ns0:c r="F34" s="111">
+        <ns0:v>108.1</ns0:v>
+      </ns0:c>
+      <ns0:c r="G34" s="53"/>
+      <ns0:c r="H34" s="53"/>
+      <ns0:c r="I34" s="5">
+        <ns0:f t="shared" ref="I34:I62" si="2">AVERAGE($E32:$E34)^12/100^11-100</ns0:f>
+        <ns0:v>5.4936577073865607</ns0:v>
+      </ns0:c>
+      <ns0:c r="J34" s="8"/>
+      <ns0:c r="K34" s="8"/>
+      <ns0:c r="L34" s="8"/>
+      <ns0:c r="M34" s="8"/>
+    </ns0:row>
+    <ns0:row r="35" spans="1:13" ht="14.25" customHeight="1" ns3:dyDescent="0.3">
+      <ns0:c r="A35" s="46">
+        <ns0:v>45536</ns0:v>
+      </ns0:c>
+      <ns0:c r="B35" s="53"/>
+      <ns0:c r="C35" s="53"/>
+      <ns0:c r="D35" s="53"/>
+      <ns0:c r="E35" s="112">
+        <ns0:v>100.62</ns0:v>
+      </ns0:c>
+      <ns0:c r="F35" s="111">
+        <ns0:v>106.91</ns0:v>
+      </ns0:c>
+      <ns0:c r="G35" s="53"/>
+      <ns0:c r="H35" s="53"/>
+      <ns0:c r="I35" s="5">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>7.3570066212323866</ns0:v>
+      </ns0:c>
+      <ns0:c r="J35" s="8"/>
+      <ns0:c r="K35" s="8"/>
+      <ns0:c r="L35" s="8"/>
+      <ns0:c r="M35" s="8"/>
+    </ns0:row>
+    <ns0:row r="36" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A36" s="49">
+        <ns0:v>45566</ns0:v>
+      </ns0:c>
+      <ns0:c r="B36" s="53"/>
+      <ns0:c r="C36" s="53"/>
+      <ns0:c r="D36" s="53"/>
+      <ns0:c r="E36" s="113">
+        <ns0:v>101.02</ns0:v>
+      </ns0:c>
+      <ns0:c r="F36" s="111">
+        <ns0:v>107.49</ns0:v>
+      </ns0:c>
+      <ns0:c r="G36" s="53"/>
+      <ns0:c r="H36" s="53"/>
+      <ns0:c r="I36" s="5">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>7.1437534623089078</ns0:v>
+      </ns0:c>
+      <ns0:c r="J36" s="8"/>
+      <ns0:c r="K36" s="8"/>
+      <ns0:c r="L36" s="8"/>
+      <ns0:c r="M36" s="8"/>
+    </ns0:row>
+    <ns0:row r="37" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A37" s="64">
+        <ns0:v>45597</ns0:v>
+      </ns0:c>
+      <ns0:c r="B37" s="65"/>
+      <ns0:c r="C37" s="65"/>
+      <ns0:c r="D37" s="65"/>
+      <ns0:c r="E37" s="114">
+        <ns0:v>101.5</ns0:v>
+      </ns0:c>
+      <ns0:c r="F37" s="115">
+        <ns0:v>108.31</ns0:v>
+      </ns0:c>
+      <ns0:c r="G37" s="65"/>
+      <ns0:c r="H37" s="65"/>
+      <ns0:c r="I37" s="5">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>13.308867445393446</ns0:v>
+      </ns0:c>
+      <ns0:c r="J37" s="8"/>
+      <ns0:c r="K37" s="8"/>
+      <ns0:c r="L37" s="8"/>
+      <ns0:c r="M37" s="8"/>
+    </ns0:row>
+    <ns0:row r="38" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A38" s="49">
+        <ns0:v>45627</ns0:v>
+      </ns0:c>
+      <ns0:c r="B38" s="57"/>
+      <ns0:c r="C38" s="57"/>
+      <ns0:c r="D38" s="57"/>
+      <ns0:c r="E38" s="113">
+        <ns0:v>100.91</ns0:v>
+      </ns0:c>
+      <ns0:c r="F38" s="111">
+        <ns0:v>108.98</ns0:v>
+      </ns0:c>
+      <ns0:c r="G38" s="62"/>
+      <ns0:c r="H38" s="57"/>
+      <ns0:c r="I38" s="53">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>14.616501588558791</ns0:v>
+      </ns0:c>
+      <ns0:c r="J38" s="8"/>
+      <ns0:c r="K38" s="8"/>
+      <ns0:c r="L38" s="8"/>
+      <ns0:c r="M38" s="8"/>
+    </ns0:row>
+    <ns0:row r="39" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A39" s="59">
+        <ns0:v>45658</ns0:v>
+      </ns0:c>
+      <ns0:c r="B39" s="55"/>
+      <ns0:c r="C39" s="55"/>
+      <ns0:c r="D39" s="55"/>
+      <ns0:c r="E39" s="113">
+        <ns0:v>100.84</ns0:v>
+      </ns0:c>
+      <ns0:c r="F39" s="113">
+        <ns0:v>108.95</ns0:v>
+      </ns0:c>
+      <ns0:c r="G39" s="62"/>
+      <ns0:c r="H39" s="62"/>
+      <ns0:c r="I39" s="55">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>13.803248161387785</ns0:v>
+      </ns0:c>
+      <ns0:c r="J39" s="7"/>
+      <ns0:c r="K39" s="7"/>
+      <ns0:c r="L39" s="7"/>
+      <ns0:c r="M39" s="7"/>
+    </ns0:row>
+    <ns0:row r="40" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A40" s="60">
+        <ns0:v>45689</ns0:v>
+      </ns0:c>
+      <ns0:c r="B40" s="55"/>
+      <ns0:c r="C40" s="55"/>
+      <ns0:c r="D40" s="55"/>
+      <ns0:c r="E40" s="113">
+        <ns0:v>101.34</ns0:v>
+      </ns0:c>
+      <ns0:c r="F40" s="113">
+        <ns0:v>109.83</ns0:v>
+      </ns0:c>
+      <ns0:c r="G40" s="62"/>
+      <ns0:c r="H40" s="62"/>
+      <ns0:c r="I40" s="55">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>13.084800413622574</ns0:v>
+      </ns0:c>
+      <ns0:c r="J40" s="7"/>
+      <ns0:c r="K40" s="7"/>
+      <ns0:c r="L40" s="7"/>
+      <ns0:c r="M40" s="7"/>
+    </ns0:row>
+    <ns0:row r="41" spans="1:13" ht="15" thickBot="1" ns3:dyDescent="0.35">
+      <ns0:c r="A41" s="71">
+        <ns0:v>45717</ns0:v>
+      </ns0:c>
+      <ns0:c r="B41" s="66"/>
+      <ns0:c r="C41" s="66"/>
+      <ns0:c r="D41" s="66"/>
+      <ns0:c r="E41" s="114">
+        <ns0:v>100.81</ns0:v>
+      </ns0:c>
+      <ns0:c r="F41" s="114">
+        <ns0:v>110.13</ns0:v>
+      </ns0:c>
+      <ns0:c r="G41" s="72"/>
+      <ns0:c r="H41" s="72"/>
+      <ns0:c r="I41" s="66">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>12.637884379001619</ns0:v>
+      </ns0:c>
+      <ns0:c r="J41" s="7"/>
+      <ns0:c r="K41" s="7"/>
+      <ns0:c r="L41" s="7"/>
+      <ns0:c r="M41" s="7"/>
+    </ns0:row>
+    <ns0:row r="42" spans="1:13" ht="15" thickBot="1" ns3:dyDescent="0.35">
+      <ns0:c r="A42" s="78">
+        <ns0:v>45748</ns0:v>
+      </ns0:c>
+      <ns0:c r="B42" s="79"/>
+      <ns0:c r="C42" s="79"/>
+      <ns0:c r="D42" s="79"/>
+      <ns0:c r="E42" s="116">
+        <ns0:v>100.53</ns0:v>
+      </ns0:c>
+      <ns0:c r="F42" s="116">
+        <ns0:v>110.3</ns0:v>
+      </ns0:c>
+      <ns0:c r="G42" s="80"/>
+      <ns0:c r="H42" s="80"/>
+      <ns0:c r="I42" s="79">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>11.262713373249582</ns0:v>
+      </ns0:c>
+      <ns0:c r="J42" s="7"/>
+      <ns0:c r="K42" s="7"/>
+      <ns0:c r="L42" s="7"/>
+      <ns0:c r="M42" s="7"/>
+    </ns0:row>
+    <ns0:row r="43" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A43" s="74">
+        <ns0:v>45778</ns0:v>
+      </ns0:c>
+      <ns0:c r="B43" s="75"/>
+      <ns0:c r="C43" s="75"/>
+      <ns0:c r="D43" s="75"/>
+      <ns0:c r="E43" s="117">
+        <ns0:v>99.93</ns0:v>
+      </ns0:c>
+      <ns0:c r="F43" s="117">
+        <ns0:v>109.2</ns0:v>
+      </ns0:c>
+      <ns0:c r="G43" s="76"/>
+      <ns0:c r="H43" s="76"/>
+      <ns0:c r="I43" s="75">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>5.1999643920905925</ns0:v>
+      </ns0:c>
+      <ns0:c r="J43" s="7"/>
+      <ns0:c r="K43" s="7"/>
+      <ns0:c r="L43" s="7"/>
+      <ns0:c r="M43" s="7"/>
+    </ns0:row>
+    <ns0:row r="44" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A44" s="60">
+        <ns0:v>45809</ns0:v>
+      </ns0:c>
+      <ns0:c r="B44" s="55"/>
+      <ns0:c r="C44" s="55"/>
+      <ns0:c r="D44" s="55"/>
+      <ns0:c r="E44" s="113">
+        <ns0:v>99.96</ns0:v>
+      </ns0:c>
+      <ns0:c r="F44" s="113">
+        <ns0:v>108.96</ns0:v>
+      </ns0:c>
+      <ns0:c r="G44" s="62"/>
+      <ns0:c r="H44" s="62"/>
+      <ns0:c r="I44" s="55">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>1.6929965585858326</ns0:v>
+      </ns0:c>
+      <ns0:c r="J44" s="7"/>
+      <ns0:c r="K44" s="7"/>
+      <ns0:c r="L44" s="7"/>
+      <ns0:c r="M44" s="7"/>
+    </ns0:row>
+    <ns0:row r="45" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A45" s="59">
+        <ns0:v>45839</ns0:v>
+      </ns0:c>
+      <ns0:c r="B45" s="55"/>
+      <ns0:c r="C45" s="55"/>
+      <ns0:c r="D45" s="55"/>
+      <ns0:c r="E45" s="113">
+        <ns0:v>100.36</ns0:v>
+      </ns0:c>
+      <ns0:c r="F45" s="113">
+        <ns0:v>108.19</ns0:v>
+      </ns0:c>
+      <ns0:c r="G45" s="62"/>
+      <ns0:c r="H45" s="62"/>
+      <ns0:c r="I45" s="55">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>1.0045960887180883</ns0:v>
+      </ns0:c>
+      <ns0:c r="J45" s="5"/>
+      <ns0:c r="K45" s="5"/>
+      <ns0:c r="L45" s="5"/>
+      <ns0:c r="M45" s="5"/>
+    </ns0:row>
+    <ns0:row r="46" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A46" s="60">
+        <ns0:v>45870</ns0:v>
+      </ns0:c>
+      <ns0:c r="B46" s="55"/>
+      <ns0:c r="C46" s="55"/>
+      <ns0:c r="D46" s="55"/>
+      <ns0:c r="E46" s="113">
+        <ns0:v>99.43</ns0:v>
+      </ns0:c>
+      <ns0:c r="F46" s="113">
+        <ns0:v>107.48</ns0:v>
+      </ns0:c>
+      <ns0:c r="G46" s="62"/>
+      <ns0:c r="H46" s="62"/>
+      <ns0:c r="I46" s="55">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>-0.99542937430834399</ns0:v>
+      </ns0:c>
+      <ns0:c r="J46" s="5"/>
+      <ns0:c r="K46" s="5"/>
+      <ns0:c r="L46" s="5"/>
+      <ns0:c r="M46" s="5"/>
+    </ns0:row>
+    <ns0:row r="47" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A47" s="59">
+        <ns0:v>45901</ns0:v>
+      </ns0:c>
+      <ns0:c r="B47" s="55"/>
+      <ns0:c r="C47" s="55"/>
+      <ns0:c r="D47" s="55"/>
+      <ns0:c r="E47" s="113">
+        <ns0:v>101</ns0:v>
+      </ns0:c>
+      <ns0:c r="F47" s="113">
+        <ns0:v>107.88</ns0:v>
+      </ns0:c>
+      <ns0:c r="G47" s="62"/>
+      <ns0:c r="H47" s="62"/>
+      <ns0:c r="I47" s="55">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>3.2061714591574031</ns0:v>
+      </ns0:c>
+      <ns0:c r="J47" s="5"/>
+      <ns0:c r="K47" s="5"/>
+      <ns0:c r="L47" s="5"/>
+      <ns0:c r="M47" s="5"/>
+    </ns0:row>
+    <ns0:row r="48" spans="1:13" ht="18.45" customHeight="1" ns3:dyDescent="0.3">
+      <ns0:c r="A48" s="60">
+        <ns0:v>45931</ns0:v>
+      </ns0:c>
+      <ns0:c r="B48" s="55"/>
+      <ns0:c r="C48" s="55"/>
+      <ns0:c r="D48" s="55"/>
+      <ns0:c r="E48" s="113">
+        <ns0:v>100.53</ns0:v>
+      </ns0:c>
+      <ns0:c r="F48" s="113">
+        <ns0:v>107.36</ns0:v>
+      </ns0:c>
+      <ns0:c r="G48" s="62"/>
+      <ns0:c r="H48" s="62"/>
+      <ns0:c r="I48" s="55">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>3.9083101131258928</ns0:v>
+      </ns0:c>
+      <ns0:c r="J48" s="5"/>
+      <ns0:c r="K48" s="5"/>
+      <ns0:c r="L48" s="5"/>
+      <ns0:c r="M48" s="5"/>
+    </ns0:row>
+    <ns0:row r="49" spans="1:13" ht="15" thickBot="1" ns3:dyDescent="0.35">
+      <ns0:c r="A49" s="71">
+        <ns0:v>45962</ns0:v>
+      </ns0:c>
+      <ns0:c r="B49" s="66"/>
+      <ns0:c r="C49" s="55"/>
+      <ns0:c r="D49" s="55"/>
+      <ns0:c r="E49" s="114">
+        <ns0:v>100.15</ns0:v>
+      </ns0:c>
+      <ns0:c r="F49" s="114">
+        <ns0:v>105.93</ns0:v>
+      </ns0:c>
+      <ns0:c r="G49" s="72"/>
+      <ns0:c r="H49" s="72"/>
+      <ns0:c r="I49" s="66">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>6.9308886717982716</ns0:v>
+      </ns0:c>
+      <ns0:c r="J49" s="5"/>
+      <ns0:c r="K49" s="5"/>
+      <ns0:c r="L49" s="5"/>
+      <ns0:c r="M49" s="5"/>
+    </ns0:row>
+    <ns0:row r="50" spans="1:13" ht="15" customHeight="1" thickBot="1" ns3:dyDescent="0.35">
+      <ns0:c r="A50" s="78">
+        <ns0:v>45992</ns0:v>
+      </ns0:c>
+      <ns0:c r="B50" s="79"/>
+      <ns0:c r="C50" s="55"/>
+      <ns0:c r="D50" s="55"/>
+      <ns0:c r="E50" s="116">
+        <ns0:v>100.29</ns0:v>
+      </ns0:c>
+      <ns0:c r="F50" s="116">
+        <ns0:v>105.28</ns0:v>
+      </ns0:c>
+      <ns0:c r="G50" s="80"/>
+      <ns0:c r="H50" s="80"/>
+      <ns0:c r="I50" s="79">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>3.949748431031864</ns0:v>
+      </ns0:c>
+      <ns0:c r="J50" s="5"/>
+      <ns0:c r="K50" s="5"/>
+      <ns0:c r="L50" s="5"/>
+      <ns0:c r="M50" s="5"/>
+    </ns0:row>
+    <ns0:row r="51" spans="1:13" ht="15" thickBot="1" ns3:dyDescent="0.35">
+      <ns0:c r="A51" s="74">
+        <ns0:v>46023</ns0:v>
+      </ns0:c>
+      <ns0:c r="B51" s="87"/>
+      <ns0:c r="C51" s="55">
+        <ns0:f t="shared" ref="C51:D57" si="3">E51-100</ns0:f>
+        <ns0:v>1.6</ns0:v>
+      </ns0:c>
+      <ns0:c r="D51" s="55">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>6.07</ns0:v>
+      </ns0:c>
+      <ns0:c r="E51" s="75">
+        <ns0:v>101.6</ns0:v>
+      </ns0:c>
+      <ns0:c r="F51" s="75">
+        <ns0:f t="shared" ref="F51:F74" si="4">ROUND(PRODUCT(E40:E51)/100^11,2)</ns0:f>
+        <ns0:v>106.07</ns0:v>
+      </ns0:c>
+      <ns0:c r="G51" s="118">
+        <ns0:v>101.6</ns0:v>
+      </ns0:c>
+      <ns0:c r="H51" s="118">
+        <ns0:v>106.07</ns0:v>
+      </ns0:c>
+      <ns0:c r="I51" s="79">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>8.4722085025153433</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="52" spans="1:13" ht="15" thickBot="1" ns3:dyDescent="0.35">
+      <ns0:c r="A52" s="60">
+        <ns0:v>46054</ns0:v>
+      </ns0:c>
+      <ns0:c r="B52" s="56"/>
+      <ns0:c r="C52" s="55">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>1.1</ns0:v>
+      </ns0:c>
+      <ns0:c r="D52" s="55">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>5.82</ns0:v>
+      </ns0:c>
+      <ns0:c r="E52" s="55">
+        <ns0:v>101.1</ns0:v>
+      </ns0:c>
+      <ns0:c r="F52" s="55">
+        <ns0:f t="shared" si="4"/>
+        <ns0:v>105.82</ns0:v>
+      </ns0:c>
+      <ns0:c r="G52" s="107">
+        <ns0:v>101.1</ns0:v>
+      </ns0:c>
+      <ns0:c r="H52" s="107">
+        <ns0:v>105.82</ns0:v>
+      </ns0:c>
+      <ns0:c r="I52" s="79">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>12.637884379001619</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="53" spans="1:13" ht="15" thickBot="1" ns3:dyDescent="0.35">
+      <ns0:c r="A53" s="59">
+        <ns0:v>46082</ns0:v>
+      </ns0:c>
+      <ns0:c r="B53" s="56"/>
+      <ns0:c r="C53" s="55">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>0.54</ns0:v>
+      </ns0:c>
+      <ns0:c r="D53" s="55">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>5.54</ns0:v>
+      </ns0:c>
+      <ns0:c r="E53" s="70">
+        <ns0:v>100.54</ns0:v>
+      </ns0:c>
+      <ns0:c r="F53" s="55">
+        <ns0:f t="shared" si="4"/>
+        <ns0:v>105.54</ns0:v>
+      </ns0:c>
+      <ns0:c r="G53" s="107">
+        <ns0:v>100.54</ns0:v>
+      </ns0:c>
+      <ns0:c r="H53" s="107">
+        <ns0:v>105.54</ns0:v>
+      </ns0:c>
+      <ns0:c r="I53" s="79">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>13.758222891107337</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="54" spans="1:13" ht="15" thickBot="1" ns3:dyDescent="0.35">
+      <ns0:c r="A54" s="60">
+        <ns0:v>46113</ns0:v>
+      </ns0:c>
+      <ns0:c r="B54" s="56"/>
+      <ns0:c r="C54" s="55">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>-0.28</ns0:v>
+      </ns0:c>
+      <ns0:c r="D54" s="55">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>4.69</ns0:v>
+      </ns0:c>
+      <ns0:c r="E54" s="55">
+        <ns0:v>99.72</ns0:v>
+      </ns0:c>
+      <ns0:c r="F54" s="55">
+        <ns0:f t="shared" si="4"/>
+        <ns0:v>104.69</ns0:v>
+      </ns0:c>
+      <ns0:c r="G54" s="107">
+        <ns0:v>99.72</ns0:v>
+      </ns0:c>
+      <ns0:c r="H54" s="107">
+        <ns0:v>104.69</ns0:v>
+      </ns0:c>
+      <ns0:c r="I54" s="79">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>5.5777080228274372</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="55" spans="1:13" ht="15" thickBot="1" ns3:dyDescent="0.35">
+      <ns0:c r="A55" s="59">
+        <ns0:v>46143</ns0:v>
+      </ns0:c>
+      <ns0:c r="B55" s="68"/>
+      <ns0:c r="C55" s="55">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>0.1</ns0:v>
+      </ns0:c>
+      <ns0:c r="D55" s="55">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>4.86</ns0:v>
+      </ns0:c>
+      <ns0:c r="E55" s="55">
+        <ns0:v>100.09</ns0:v>
+      </ns0:c>
+      <ns0:c r="F55" s="55">
+        <ns0:f t="shared" si="4"/>
+        <ns0:v>104.86</ns0:v>
+      </ns0:c>
+      <ns0:c r="G55" s="107">
+        <ns0:v>99.9</ns0:v>
+      </ns0:c>
+      <ns0:c r="H55" s="107">
+        <ns0:v>104.66</ns0:v>
+      </ns0:c>
+      <ns0:c r="I55" s="79">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>1.44954211884</ns0:v>
+      </ns0:c>
+      <ns0:c r="J55" s="42"/>
+      <ns0:c r="K55" s="42"/>
+      <ns0:c r="L55" s="42"/>
+      <ns0:c r="M55" s="42"/>
+    </ns0:row>
+    <ns0:row r="56" spans="1:13" ht="15" thickBot="1" ns3:dyDescent="0.35">
+      <ns0:c r="A56" s="60">
+        <ns0:v>46174</ns0:v>
+      </ns0:c>
+      <ns0:c r="B56" s="56"/>
+      <ns0:c r="C56" s="55">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>0.3</ns0:v>
+      </ns0:c>
+      <ns0:c r="D56" s="55">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>5.22</ns0:v>
+      </ns0:c>
+      <ns0:c r="E56" s="55">
+        <ns0:v>101.06</ns0:v>
+      </ns0:c>
+      <ns0:c r="F56" s="55">
+        <ns0:f t="shared" si="4"/>
+        <ns0:v>105.22</ns0:v>
+      </ns0:c>
+      <ns0:c r="G56" s="107">
+        <ns0:v>100</ns0:v>
+      </ns0:c>
+      <ns0:c r="H56" s="107">
+        <ns0:v>104.7</ns0:v>
+      </ns0:c>
+      <ns0:c r="I56" s="79">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>0.481057409268</ns0:v>
+      </ns0:c>
+      <ns0:c r="J56"/>
+      <ns0:c r="K56"/>
+      <ns0:c r="L56"/>
+      <ns0:c r="M56"/>
+    </ns0:row>
+    <ns0:row r="57" spans="1:13" ht="15" thickBot="1" ns3:dyDescent="0.35">
+      <ns0:c r="A57" s="59">
+        <ns0:v>46204</ns0:v>
+      </ns0:c>
+      <ns0:c r="B57" s="69"/>
+      <ns0:c r="C57" s="55">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>-0.15</ns0:v>
+      </ns0:c>
+      <ns0:c r="D57" s="55">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>4.69</ns0:v>
+      </ns0:c>
+      <ns0:c r="E57" s="55">
+        <ns0:v>101.70</ns0:v>
+      </ns0:c>
+      <ns0:c r="F57" s="55">
+        <ns0:f t="shared" si="4"/>
+        <ns0:v>104.69</ns0:v>
+      </ns0:c>
+      <ns0:c r="G57" s="107">
+        <ns0:v>99.9</ns0:v>
+      </ns0:c>
+      <ns0:c r="H57" s="107">
+        <ns0:v>104.22</ns0:v>
+      </ns0:c>
+      <ns0:c r="I57" s="79">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>1.00459608872</ns0:v>
+      </ns0:c>
+      <ns0:c r="J57"/>
+      <ns0:c r="K57"/>
+      <ns0:c r="L57"/>
+      <ns0:c r="M57"/>
+    </ns0:row>
+    <ns0:row r="58" spans="1:13" ht="15" thickBot="1" ns3:dyDescent="0.35">
+      <ns0:c r="A58" s="60">
+        <ns0:v>46235</ns0:v>
+      </ns0:c>
+      <ns0:c r="B58" s="69"/>
+      <ns0:c r="C58" s="69"/>
+      <ns0:c r="D58" s="69"/>
+      <ns0:c r="E58" s="70">
+        <ns0:v>100.50</ns0:v>
+      </ns0:c>
+      <ns0:c r="F58" s="55">
+        <ns0:f t="shared" si="4"/>
+        <ns0:v>105.08</ns0:v>
+      </ns0:c>
+      <ns0:c r="G58" s="107">
+        <ns0:v>99.85</ns0:v>
+      </ns0:c>
+      <ns0:c r="H58" s="107">
+        <ns0:v>104.66</ns0:v>
+      </ns0:c>
+      <ns0:c r="I58" s="79">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>-0.19981676848</ns0:v>
+      </ns0:c>
+      <ns0:c r="J58"/>
+      <ns0:c r="K58"/>
+      <ns0:c r="L58"/>
+      <ns0:c r="M58"/>
+    </ns0:row>
+    <ns0:row r="59" spans="1:13" ht="15" thickBot="1" ns3:dyDescent="0.35">
+      <ns0:c r="A59" s="59">
+        <ns0:v>46266</ns0:v>
+      </ns0:c>
+      <ns0:c r="B59" s="69"/>
+      <ns0:c r="C59" s="69"/>
+      <ns0:c r="D59" s="69"/>
+      <ns0:c r="E59" s="70">
+        <ns0:v>100.65</ns0:v>
+      </ns0:c>
+      <ns0:c r="F59" s="55">
+        <ns0:f t="shared" si="4"/>
+        <ns0:v>104.4</ns0:v>
+      </ns0:c>
+      <ns0:c r="G59" s="107">
+        <ns0:v>100.45</ns0:v>
+      </ns0:c>
+      <ns0:c r="H59" s="107">
+        <ns0:v>104.09</ns0:v>
+      </ns0:c>
+      <ns0:c r="I59" s="79">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="J59"/>
+      <ns0:c r="K59"/>
+      <ns0:c r="L59"/>
+      <ns0:c r="M59"/>
+    </ns0:row>
+    <ns0:row r="60" spans="1:13" ht="15" thickBot="1" ns3:dyDescent="0.35">
+      <ns0:c r="A60" s="60">
+        <ns0:v>46296</ns0:v>
+      </ns0:c>
+      <ns0:c r="B60" s="56"/>
+      <ns0:c r="C60" s="56"/>
+      <ns0:c r="D60" s="56"/>
+      <ns0:c r="E60" s="70">
+        <ns0:v>101.30</ns0:v>
+      </ns0:c>
+      <ns0:c r="F60" s="55">
+        <ns0:f t="shared" si="4"/>
+        <ns0:v>105.2</ns0:v>
+      </ns0:c>
+      <ns0:c r="G60" s="107">
+        <ns0:v>101.3</ns0:v>
+      </ns0:c>
+      <ns0:c r="H60" s="107">
+        <ns0:v>104.88</ns0:v>
+      </ns0:c>
+      <ns0:c r="I60" s="79">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>5.95669462245</ns0:v>
+      </ns0:c>
+      <ns0:c r="J60"/>
+      <ns0:c r="K60"/>
+      <ns0:c r="L60"/>
+      <ns0:c r="M60"/>
+    </ns0:row>
+    <ns0:row r="61" spans="1:13" ht="15" thickBot="1" ns3:dyDescent="0.35">
+      <ns0:c r="A61" s="59">
+        <ns0:v>46327</ns0:v>
+      </ns0:c>
+      <ns0:c r="B61" s="56"/>
+      <ns0:c r="C61" s="56"/>
+      <ns0:c r="D61" s="56"/>
+      <ns0:c r="E61" s="70">
+        <ns0:v>100.45</ns0:v>
+      </ns0:c>
+      <ns0:c r="F61" s="55">
+        <ns0:f t="shared" si="4"/>
+        <ns0:v>105.3</ns0:v>
+      </ns0:c>
+      <ns0:c r="G61" s="107">
+        <ns0:v>100.3</ns0:v>
+      </ns0:c>
+      <ns0:c r="H61" s="107">
+        <ns0:v>105.04</ns0:v>
+      </ns0:c>
+      <ns0:c r="I61" s="79">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>7.87040260178</ns0:v>
+      </ns0:c>
+      <ns0:c r="J61"/>
+      <ns0:c r="K61"/>
+      <ns0:c r="L61"/>
+      <ns0:c r="M61"/>
+    </ns0:row>
+    <ns0:row r="62" spans="1:13" ht="15" thickBot="1" ns3:dyDescent="0.35">
+      <ns0:c r="A62" s="60">
+        <ns0:v>46357</ns0:v>
+      </ns0:c>
+      <ns0:c r="B62" s="56"/>
+      <ns0:c r="C62" s="56"/>
+      <ns0:c r="D62" s="56"/>
+      <ns0:c r="E62" s="70">
+        <ns0:v>100.50</ns0:v>
+      </ns0:c>
+      <ns0:c r="F62" s="55">
+        <ns0:f t="shared" si="4"/>
+        <ns0:v>105.32</ns0:v>
+      </ns0:c>
+      <ns0:c r="G62" s="107">
+        <ns0:v>100.35</ns0:v>
+      </ns0:c>
+      <ns0:c r="H62" s="107">
+        <ns0:v>105.1</ns0:v>
+      </ns0:c>
+      <ns0:c r="I62" s="79">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>7.65621472911</ns0:v>
+      </ns0:c>
+      <ns0:c r="J62"/>
+      <ns0:c r="K62"/>
+      <ns0:c r="L62"/>
+      <ns0:c r="M62"/>
+    </ns0:row>
+    <ns0:row r="63" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A63" s="59">
+        <ns0:v>46388</ns0:v>
+      </ns0:c>
+      <ns0:c r="E63" s="8">
+        <ns0:v>100.90</ns0:v>
+      </ns0:c>
+      <ns0:c r="F63" s="55">
+        <ns0:f t="shared" si="4"/>
+        <ns0:v>104.64</ns0:v>
+      </ns0:c>
+      <ns0:c r="G63" s="31">
+        <ns0:v>100.95</ns0:v>
+      </ns0:c>
+      <ns0:c r="H63" s="31">
+        <ns0:v>104.43</ns0:v>
+      </ns0:c>
+      <ns0:c r="I63" s="8"/>
+      <ns0:c r="J63"/>
+      <ns0:c r="K63"/>
+      <ns0:c r="L63"/>
+      <ns0:c r="M63"/>
+    </ns0:row>
+    <ns0:row r="64" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A64" s="60">
+        <ns0:v>46419</ns0:v>
+      </ns0:c>
+      <ns0:c r="E64" s="8">
+        <ns0:v>100.65</ns0:v>
+      </ns0:c>
+      <ns0:c r="F64" s="55">
+        <ns0:f t="shared" si="4"/>
+        <ns0:v>104.18</ns0:v>
+      </ns0:c>
+      <ns0:c r="G64" s="31">
+        <ns0:v>100.65</ns0:v>
+      </ns0:c>
+      <ns0:c r="H64" s="31">
+        <ns0:v>103.97</ns0:v>
+      </ns0:c>
+      <ns0:c r="I64" s="8"/>
+      <ns0:c r="J64"/>
+      <ns0:c r="K64"/>
+      <ns0:c r="L64"/>
+      <ns0:c r="M64"/>
+    </ns0:row>
+    <ns0:row r="65" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A65" s="59">
+        <ns0:v>46447</ns0:v>
+      </ns0:c>
+      <ns0:c r="E65" s="8">
+        <ns0:v>100.50</ns0:v>
+      </ns0:c>
+      <ns0:c r="F65" s="55">
+        <ns0:f t="shared" si="4"/>
+        <ns0:v>104.13</ns0:v>
+      </ns0:c>
+      <ns0:c r="G65" s="31">
+        <ns0:v>100.5</ns0:v>
+      </ns0:c>
+      <ns0:c r="H65" s="31">
+        <ns0:v>103.93</ns0:v>
+      </ns0:c>
+      <ns0:c r="I65" s="8"/>
+      <ns0:c r="J65"/>
+      <ns0:c r="K65"/>
+      <ns0:c r="L65"/>
+      <ns0:c r="M65"/>
+    </ns0:row>
+    <ns0:row r="66" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A66" s="60">
+        <ns0:v>46478</ns0:v>
+      </ns0:c>
+      <ns0:c r="E66" s="8">
+        <ns0:v>100.45</ns0:v>
+      </ns0:c>
+      <ns0:c r="F66" s="55">
+        <ns0:f t="shared" si="4"/>
+        <ns0:v>104.9</ns0:v>
+      </ns0:c>
+      <ns0:c r="G66" s="31">
+        <ns0:v>100.45</ns0:v>
+      </ns0:c>
+      <ns0:c r="H66" s="31">
+        <ns0:v>104.69</ns0:v>
+      </ns0:c>
+      <ns0:c r="I66" s="8"/>
+      <ns0:c r="J66"/>
+      <ns0:c r="K66"/>
+      <ns0:c r="L66"/>
+      <ns0:c r="M66"/>
+    </ns0:row>
+    <ns0:row r="67" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A67" s="59">
+        <ns0:v>46508</ns0:v>
+      </ns0:c>
+      <ns0:c r="E67" s="8">
+        <ns0:v>100.20</ns0:v>
+      </ns0:c>
+      <ns0:c r="F67" s="55">
+        <ns0:f t="shared" si="4"/>
+        <ns0:v>105</ns0:v>
+      </ns0:c>
+      <ns0:c r="G67" s="31">
+        <ns0:v>100.2</ns0:v>
+      </ns0:c>
+      <ns0:c r="H67" s="31">
+        <ns0:v>105</ns0:v>
+      </ns0:c>
+      <ns0:c r="I67" s="8"/>
+      <ns0:c r="J67"/>
+      <ns0:c r="K67"/>
+      <ns0:c r="L67"/>
+      <ns0:c r="M67"/>
+    </ns0:row>
+    <ns0:row r="68" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A68" s="60">
+        <ns0:v>46539</ns0:v>
+      </ns0:c>
+      <ns0:c r="E68" s="8">
+        <ns0:v>100.15</ns0:v>
+      </ns0:c>
+      <ns0:c r="F68" s="55">
+        <ns0:f t="shared" si="4"/>
+        <ns0:v>104.79</ns0:v>
+      </ns0:c>
+      <ns0:c r="G68" s="31">
+        <ns0:v>100.1</ns0:v>
+      </ns0:c>
+      <ns0:c r="H68" s="31">
+        <ns0:v>105.11</ns0:v>
+      </ns0:c>
+      <ns0:c r="I68" s="8"/>
+      <ns0:c r="J68"/>
+      <ns0:c r="K68"/>
+      <ns0:c r="L68"/>
+      <ns0:c r="M68"/>
+    </ns0:row>
+    <ns0:row r="69" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A69" s="59">
+        <ns0:v>46569</ns0:v>
+      </ns0:c>
+      <ns0:c r="E69" s="8">
+        <ns0:v>100.05</ns0:v>
+      </ns0:c>
+      <ns0:c r="F69" s="55">
+        <ns0:f t="shared" si="4"/>
+        <ns0:v>105</ns0:v>
+      </ns0:c>
+      <ns0:c r="G69" s="31">
+        <ns0:v>100.05</ns0:v>
+      </ns0:c>
+      <ns0:c r="H69" s="31">
+        <ns0:v>105.26</ns0:v>
+      </ns0:c>
+      <ns0:c r="I69" s="8"/>
+      <ns0:c r="J69"/>
+      <ns0:c r="K69"/>
+      <ns0:c r="L69"/>
+      <ns0:c r="M69"/>
+    </ns0:row>
+    <ns0:row r="70" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A70" s="60">
+        <ns0:v>46600</ns0:v>
+      </ns0:c>
+      <ns0:c r="E70" s="8">
+        <ns0:v>99.95</ns0:v>
+      </ns0:c>
+      <ns0:c r="F70" s="55">
+        <ns0:f t="shared" si="4"/>
+        <ns0:v>105.16</ns0:v>
+      </ns0:c>
+      <ns0:c r="G70" s="31">
+        <ns0:v>99.95</ns0:v>
+      </ns0:c>
+      <ns0:c r="H70" s="31">
+        <ns0:v>105.37</ns0:v>
+      </ns0:c>
+      <ns0:c r="I70" s="8"/>
+      <ns0:c r="J70"/>
+      <ns0:c r="K70"/>
+      <ns0:c r="L70"/>
+      <ns0:c r="M70"/>
+    </ns0:row>
+    <ns0:row r="71" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A71" s="59">
+        <ns0:v>46631</ns0:v>
+      </ns0:c>
+      <ns0:c r="E71" s="8">
+        <ns0:v>100.45</ns0:v>
+      </ns0:c>
+      <ns0:c r="F71" s="55">
+        <ns0:f t="shared" si="4"/>
+        <ns0:v>105.26</ns0:v>
+      </ns0:c>
+      <ns0:c r="G71" s="31">
+        <ns0:v>100.45</ns0:v>
+      </ns0:c>
+      <ns0:c r="H71" s="31">
+        <ns0:v>105.37</ns0:v>
+      </ns0:c>
+      <ns0:c r="I71" s="8"/>
+      <ns0:c r="J71"/>
+      <ns0:c r="K71"/>
+      <ns0:c r="L71"/>
+      <ns0:c r="M71"/>
+    </ns0:row>
+    <ns0:row r="72" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A72" s="60">
+        <ns0:v>46661</ns0:v>
+      </ns0:c>
+      <ns0:c r="E72" s="8">
+        <ns0:v>100.45</ns0:v>
+      </ns0:c>
+      <ns0:c r="F72" s="55">
+        <ns0:f t="shared" si="4"/>
+        <ns0:v>104.38</ns0:v>
+      </ns0:c>
+      <ns0:c r="G72" s="31">
+        <ns0:v>100.45</ns0:v>
+      </ns0:c>
+      <ns0:c r="H72" s="31">
+        <ns0:v>104.49</ns0:v>
+      </ns0:c>
+      <ns0:c r="I72" s="8"/>
+      <ns0:c r="J72"/>
+      <ns0:c r="K72"/>
+      <ns0:c r="L72"/>
+      <ns0:c r="M72"/>
+    </ns0:row>
+    <ns0:row r="73" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A73" s="59">
+        <ns0:v>46692</ns0:v>
+      </ns0:c>
+      <ns0:c r="E73" s="8">
+        <ns0:v>100.2</ns0:v>
+      </ns0:c>
+      <ns0:c r="F73" s="55">
+        <ns0:f t="shared" si="4"/>
+        <ns0:v>104.33</ns0:v>
+      </ns0:c>
+      <ns0:c r="G73" s="31">
+        <ns0:v>100.2</ns0:v>
+      </ns0:c>
+      <ns0:c r="H73" s="31">
+        <ns0:v>104.38</ns0:v>
+      </ns0:c>
+      <ns0:c r="I73" s="8"/>
+      <ns0:c r="J73"/>
+      <ns0:c r="K73"/>
+      <ns0:c r="L73"/>
+      <ns0:c r="M73"/>
+    </ns0:row>
+    <ns0:row r="74" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A74" s="60">
+        <ns0:v>46722</ns0:v>
+      </ns0:c>
+      <ns0:c r="E74" s="8">
+        <ns0:v>100</ns0:v>
+      </ns0:c>
+      <ns0:c r="F74" s="55">
+        <ns0:f t="shared" si="4"/>
+        <ns0:v>104.02</ns0:v>
+      </ns0:c>
+      <ns0:c r="G74" s="31">
+        <ns0:v>100</ns0:v>
+      </ns0:c>
+      <ns0:c r="H74" s="31">
+        <ns0:v>104.02</ns0:v>
+      </ns0:c>
+      <ns0:c r="I74" s="8"/>
+      <ns0:c r="J74"/>
+      <ns0:c r="K74"/>
+      <ns0:c r="L74"/>
+      <ns0:c r="M74"/>
+    </ns0:row>
+    <ns0:row r="75" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A75" s="40"/>
+      <ns0:c r="E75" s="22"/>
+      <ns0:c r="F75" s="8"/>
+      <ns0:c r="G75" s="31"/>
+      <ns0:c r="H75" s="31"/>
+      <ns0:c r="I75" s="8"/>
+      <ns0:c r="J75"/>
+      <ns0:c r="K75"/>
+      <ns0:c r="L75"/>
+      <ns0:c r="M75"/>
+    </ns0:row>
+    <ns0:row r="76" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A76" s="40"/>
+      <ns0:c r="E76" s="22"/>
+      <ns0:c r="F76" s="8"/>
+      <ns0:c r="G76" s="31"/>
+      <ns0:c r="H76" s="31"/>
+      <ns0:c r="I76" s="8"/>
+      <ns0:c r="J76"/>
+      <ns0:c r="K76"/>
+      <ns0:c r="L76"/>
+      <ns0:c r="M76"/>
+    </ns0:row>
+    <ns0:row r="77" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A77" s="40"/>
+      <ns0:c r="E77" s="22"/>
+      <ns0:c r="F77" s="8"/>
+      <ns0:c r="G77" s="31"/>
+      <ns0:c r="H77" s="31"/>
+      <ns0:c r="I77" s="8"/>
+      <ns0:c r="J77"/>
+      <ns0:c r="K77"/>
+      <ns0:c r="L77"/>
+      <ns0:c r="M77"/>
+    </ns0:row>
+    <ns0:row r="78" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A78" s="40"/>
+      <ns0:c r="E78" s="22"/>
+      <ns0:c r="F78" s="8"/>
+      <ns0:c r="G78" s="31"/>
+      <ns0:c r="H78" s="31"/>
+      <ns0:c r="I78" s="8"/>
+      <ns0:c r="J78"/>
+      <ns0:c r="K78"/>
+      <ns0:c r="L78"/>
+      <ns0:c r="M78"/>
+    </ns0:row>
+    <ns0:row r="79" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A79" s="40"/>
+      <ns0:c r="E79" s="22"/>
+      <ns0:c r="F79" s="8"/>
+      <ns0:c r="G79" s="31"/>
+      <ns0:c r="H79" s="31"/>
+      <ns0:c r="I79" s="8"/>
+      <ns0:c r="J79"/>
+      <ns0:c r="K79"/>
+      <ns0:c r="L79"/>
+      <ns0:c r="M79"/>
+    </ns0:row>
+    <ns0:row r="80" spans="1:13" ns3:dyDescent="0.3">
+      <ns0:c r="A80"/>
+    </ns0:row>
+    <ns0:row r="81" spans="7:13" ns3:dyDescent="0.3">
+      <ns0:c r="G81" s="5"/>
+      <ns0:c r="H81" s="5"/>
+      <ns0:c r="J81"/>
+      <ns0:c r="K81"/>
+      <ns0:c r="L81"/>
+      <ns0:c r="M81"/>
+    </ns0:row>
+    <ns0:row r="82" spans="7:13" ns3:dyDescent="0.3">
+      <ns0:c r="G82" s="5"/>
+      <ns0:c r="H82" s="5"/>
+      <ns0:c r="J82"/>
+      <ns0:c r="K82"/>
+      <ns0:c r="L82"/>
+      <ns0:c r="M82"/>
+    </ns0:row>
+    <ns0:row r="83" spans="7:13" ns3:dyDescent="0.3">
+      <ns0:c r="J83"/>
+      <ns0:c r="K83"/>
+      <ns0:c r="L83"/>
+      <ns0:c r="M83"/>
+    </ns0:row>
+    <ns0:row r="84" spans="7:13" ns3:dyDescent="0.3">
+      <ns0:c r="J84"/>
+      <ns0:c r="K84"/>
+      <ns0:c r="L84"/>
+      <ns0:c r="M84"/>
+    </ns0:row>
+    <ns0:row r="85" spans="7:13" ns3:dyDescent="0.3">
+      <ns0:c r="J85"/>
+      <ns0:c r="K85"/>
+      <ns0:c r="L85"/>
+      <ns0:c r="M85"/>
+    </ns0:row>
+    <ns0:row r="86" spans="7:13" ns3:dyDescent="0.3">
+      <ns0:c r="J86"/>
+      <ns0:c r="K86"/>
+      <ns0:c r="L86"/>
+      <ns0:c r="M86"/>
+    </ns0:row>
+    <ns0:row r="87" spans="7:13" ns3:dyDescent="0.3">
+      <ns0:c r="J87"/>
+      <ns0:c r="K87"/>
+      <ns0:c r="L87"/>
+      <ns0:c r="M87"/>
+    </ns0:row>
+    <ns0:row r="88" spans="7:13" ns3:dyDescent="0.3">
+      <ns0:c r="J88"/>
+      <ns0:c r="K88"/>
+      <ns0:c r="L88"/>
+      <ns0:c r="M88"/>
+    </ns0:row>
+    <ns0:row r="89" spans="7:13" ns3:dyDescent="0.3">
+      <ns0:c r="J89"/>
+      <ns0:c r="K89"/>
+      <ns0:c r="L89"/>
+      <ns0:c r="M89"/>
+    </ns0:row>
+    <ns0:row r="90" spans="7:13" ns3:dyDescent="0.3">
+      <ns0:c r="J90"/>
+      <ns0:c r="K90"/>
+      <ns0:c r="L90"/>
+      <ns0:c r="M90"/>
+    </ns0:row>
+    <ns0:row r="91" spans="7:13" ns3:dyDescent="0.3">
+      <ns0:c r="J91"/>
+      <ns0:c r="K91"/>
+      <ns0:c r="L91"/>
+      <ns0:c r="M91"/>
+    </ns0:row>
+    <ns0:row r="92" spans="7:13" ns3:dyDescent="0.3">
+      <ns0:c r="J92"/>
+      <ns0:c r="K92"/>
+      <ns0:c r="L92"/>
+      <ns0:c r="M92"/>
+    </ns0:row>
+    <ns0:row r="93" spans="7:13" ns3:dyDescent="0.3">
+      <ns0:c r="J93"/>
+      <ns0:c r="K93"/>
+      <ns0:c r="L93"/>
+      <ns0:c r="M93"/>
+    </ns0:row>
+  </ns0:sheetData>
+  <ns0:conditionalFormatting sqref="J23:M24">
+    <ns0:cfRule type="colorScale" priority="20">
+      <ns0:colorScale>
+        <ns0:cfvo type="min"/>
+        <ns0:cfvo type="percentile" val="50"/>
+        <ns0:cfvo type="max"/>
+        <ns0:color rgb="FF63BE7B"/>
+        <ns0:color rgb="FFFCFCFF"/>
+        <ns0:color rgb="FFF8696B"/>
+      </ns0:colorScale>
+    </ns0:cfRule>
+  </ns0:conditionalFormatting>
+  <ns0:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ns0:pageSetup paperSize="9" orientation="landscape" ns4:id="rId1"/>
+</ns0:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>